<commit_message>
Add CAT 2 daily itemized labor grid to client Excel package
Staff / Foremen / Direct / Support now emit Nathan-style date columns from L, 7-row HC / HPS / ST / OT / DT / PD blocks, and DAYSHIFT / NIGHTSHIFT. ST/OT/DT are WEEKDAY formulas. PD $ stays off Labor TM $. No Laydown sheet. Regenerated Look samples.

Co-authored-by: robertmhenderson582-ops <robertmhenderson582-ops@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/look-samples/v151_2027_aromatics_client_package.xlsx
+++ b/look-samples/v151_2027_aromatics_client_package.xlsx
@@ -30,14 +30,14 @@
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'ORG Chart'!$6:$6</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="2">'Slicer Hrs'!$A1:$E8</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="2">'Slicer Hrs'!$6:$6</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="3">'Staff'!$A1:$P9</definedName>
-    <definedName name="_xlnm.Print_Titles" localSheetId="3">'Staff'!$6:$6</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="4">'Foremen'!$A1:$P8</definedName>
-    <definedName name="_xlnm.Print_Titles" localSheetId="4">'Foremen'!$6:$6</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="5">'Direct'!$A1:$P8</definedName>
-    <definedName name="_xlnm.Print_Titles" localSheetId="5">'Direct'!$6:$6</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="6">'Support'!$A1:$P8</definedName>
-    <definedName name="_xlnm.Print_Titles" localSheetId="6">'Support'!$6:$6</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="3">'Staff'!$A1:$R21</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="3">'Staff'!$A:$K,'Staff'!$6:$6</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="4">'Foremen'!$A1:$R14</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="4">'Foremen'!$A:$K,'Foremen'!$6:$6</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="5">'Direct'!$A1:$R14</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="5">'Direct'!$A:$K,'Direct'!$6:$6</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="6">'Support'!$A1:$R14</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="6">'Support'!$A:$K,'Support'!$6:$6</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="7">'Equipment Rental'!$A1:$H8</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="7">'Equipment Rental'!$6:$6</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="8">'Tensioning Torquing equipment'!$A1:$H8</definedName>
@@ -60,7 +60,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="275" uniqueCount="93">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="295" uniqueCount="96">
   <si>
     <t>HIT SQUAD / PROJECT CONTROLS</t>
   </si>
@@ -200,155 +200,165 @@
     <t>TOTAL</t>
   </si>
   <si>
-    <t>Headcount</t>
+    <t>Total Billable</t>
+  </si>
+  <si>
+    <t>Sub Total $</t>
+  </si>
+  <si>
+    <t>Rate</t>
+  </si>
+  <si>
+    <t>Type</t>
   </si>
   <si>
     <t>PD Days</t>
   </si>
   <si>
-    <t>ST Rate</t>
-  </si>
-  <si>
-    <t>OT Rate</t>
-  </si>
-  <si>
-    <t>DT Rate</t>
+    <t>DAYSHIFT</t>
+  </si>
+  <si>
+    <t>HC</t>
+  </si>
+  <si>
+    <t>Enter Hours Per shift Here</t>
+  </si>
+  <si>
+    <t>HPS</t>
+  </si>
+  <si>
+    <t>ST</t>
+  </si>
+  <si>
+    <t>OT</t>
+  </si>
+  <si>
+    <t>DT</t>
+  </si>
+  <si>
+    <t>PD</t>
+  </si>
+  <si>
+    <t>Boilermaker Journeyman</t>
+  </si>
+  <si>
+    <t>Fire Watch</t>
+  </si>
+  <si>
+    <t>Item</t>
+  </si>
+  <si>
+    <t>Period</t>
+  </si>
+  <si>
+    <t>Qty</t>
+  </si>
+  <si>
+    <t>Periods</t>
+  </si>
+  <si>
+    <t>Rate $</t>
+  </si>
+  <si>
+    <t>Freight $</t>
+  </si>
+  <si>
+    <t>Cost $</t>
+  </si>
+  <si>
+    <t>Total $</t>
+  </si>
+  <si>
+    <t>450amp diesel welder</t>
+  </si>
+  <si>
+    <t>daily</t>
+  </si>
+  <si>
+    <t>Hydraulic tensioner</t>
+  </si>
+  <si>
+    <t>Carry deck crane</t>
+  </si>
+  <si>
+    <t>Vendor</t>
+  </si>
+  <si>
+    <t>Scope</t>
+  </si>
+  <si>
+    <t>Affiliate</t>
+  </si>
+  <si>
+    <t>Markup $</t>
+  </si>
+  <si>
+    <t>O&amp;M Crane</t>
+  </si>
+  <si>
+    <t>crane lift</t>
+  </si>
+  <si>
+    <t>No</t>
+  </si>
+  <si>
+    <t>AIR MOVER</t>
+  </si>
+  <si>
+    <t>Kind</t>
+  </si>
+  <si>
+    <t>Travelers</t>
+  </si>
+  <si>
+    <t>Miles</t>
+  </si>
+  <si>
+    <t>$ / mile</t>
+  </si>
+  <si>
+    <t>Staff</t>
+  </si>
+  <si>
+    <t>Description</t>
+  </si>
+  <si>
+    <t>Each $</t>
+  </si>
+  <si>
+    <t>Alloy rod</t>
+  </si>
+  <si>
+    <t>Stainless</t>
+  </si>
+  <si>
+    <t>Craft</t>
+  </si>
+  <si>
+    <t>COMP BW $</t>
+  </si>
+  <si>
+    <t>ST Bill $</t>
+  </si>
+  <si>
+    <t>OT Bill $</t>
+  </si>
+  <si>
+    <t>DT Bill $</t>
   </si>
   <si>
     <t>PD Rate</t>
-  </si>
-  <si>
-    <t>ST $</t>
-  </si>
-  <si>
-    <t>OT $</t>
-  </si>
-  <si>
-    <t>DT $</t>
-  </si>
-  <si>
-    <t>PD $</t>
-  </si>
-  <si>
-    <t>Total $</t>
-  </si>
-  <si>
-    <t>MH</t>
-  </si>
-  <si>
-    <t>Boilermaker Journeyman</t>
-  </si>
-  <si>
-    <t>Fire Watch</t>
-  </si>
-  <si>
-    <t>Item</t>
-  </si>
-  <si>
-    <t>Period</t>
-  </si>
-  <si>
-    <t>Qty</t>
-  </si>
-  <si>
-    <t>Periods</t>
-  </si>
-  <si>
-    <t>Rate $</t>
-  </si>
-  <si>
-    <t>Freight $</t>
-  </si>
-  <si>
-    <t>Cost $</t>
-  </si>
-  <si>
-    <t>450amp diesel welder</t>
-  </si>
-  <si>
-    <t>daily</t>
-  </si>
-  <si>
-    <t>Hydraulic tensioner</t>
-  </si>
-  <si>
-    <t>Carry deck crane</t>
-  </si>
-  <si>
-    <t>Vendor</t>
-  </si>
-  <si>
-    <t>Scope</t>
-  </si>
-  <si>
-    <t>Affiliate</t>
-  </si>
-  <si>
-    <t>Markup $</t>
-  </si>
-  <si>
-    <t>O&amp;M Crane</t>
-  </si>
-  <si>
-    <t>crane lift</t>
-  </si>
-  <si>
-    <t>No</t>
-  </si>
-  <si>
-    <t>AIR MOVER</t>
-  </si>
-  <si>
-    <t>Kind</t>
-  </si>
-  <si>
-    <t>Travelers</t>
-  </si>
-  <si>
-    <t>Miles</t>
-  </si>
-  <si>
-    <t>$ / mile</t>
-  </si>
-  <si>
-    <t>Staff</t>
-  </si>
-  <si>
-    <t>Description</t>
-  </si>
-  <si>
-    <t>Each $</t>
-  </si>
-  <si>
-    <t>Alloy rod</t>
-  </si>
-  <si>
-    <t>Stainless</t>
-  </si>
-  <si>
-    <t>Craft</t>
-  </si>
-  <si>
-    <t>COMP BW $</t>
-  </si>
-  <si>
-    <t>ST Bill $</t>
-  </si>
-  <si>
-    <t>OT Bill $</t>
-  </si>
-  <si>
-    <t>DT Bill $</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <numFmts count="3">
+  <numFmts count="4">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD"/>
     <numFmt numFmtId="165" formatCode="$#,##0.00"/>
     <numFmt numFmtId="166" formatCode="#,##0.0"/>
+    <numFmt numFmtId="167" formatCode="D-MMM"/>
   </numFmts>
   <fonts count="9" x14ac:knownFonts="1">
     <font>
@@ -405,7 +415,7 @@
       <name val="Calibri"/>
     </font>
   </fonts>
-  <fills count="7">
+  <fills count="8">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -435,6 +445,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFFF3D6"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFF8E6"/>
       </patternFill>
     </fill>
   </fills>
@@ -468,7 +483,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="25">
+  <cellXfs count="31">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -505,8 +520,16 @@
     <xf numFmtId="3" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="3" fontId="4" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="166" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="167" fontId="6" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="166" fontId="8" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="165" fontId="8" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="4" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="3" fontId="4" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="166" fontId="4" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="165" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="166" fontId="4" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="165" fontId="4" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -890,7 +913,7 @@
         <v>4</v>
       </c>
       <c r="B5" s="6">
-        <v>46269.695648078705</v>
+        <v>46269.70988202546</v>
       </c>
     </row>
     <row r="6" ht="20" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
@@ -909,10 +932,10 @@
         <v>8</v>
       </c>
       <c r="B7" s="9">
-        <f>Staff!O9</f>
+        <f>Staff!K21</f>
       </c>
       <c r="C7" s="10">
-        <f>Staff!P9</f>
+        <f>Staff!B21</f>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
@@ -920,10 +943,10 @@
         <v>9</v>
       </c>
       <c r="B8" s="12">
-        <f>Foremen!O8</f>
+        <f>Foremen!K14</f>
       </c>
       <c r="C8" s="13">
-        <f>Foremen!P8</f>
+        <f>Foremen!B14</f>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
@@ -931,10 +954,10 @@
         <v>10</v>
       </c>
       <c r="B9" s="9">
-        <f>Direct!O8</f>
+        <f>Direct!K14</f>
       </c>
       <c r="C9" s="10">
-        <f>Direct!P8</f>
+        <f>Direct!B14</f>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
@@ -942,10 +965,10 @@
         <v>11</v>
       </c>
       <c r="B10" s="12">
-        <f>Support!O8</f>
+        <f>Support!K14</f>
       </c>
       <c r="C10" s="13">
-        <f>Support!P8</f>
+        <f>Support!B14</f>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
@@ -964,7 +987,7 @@
         <v>13</v>
       </c>
       <c r="B12" s="12">
-        <f>SUM(Staff!N9,Foremen!N8,Direct!N8,Support!N8)</f>
+        <f>SUM(Staff!D21,Foremen!D14,Direct!D14,Support!D14)</f>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.25">
@@ -1036,7 +1059,7 @@
         <v>22</v>
       </c>
       <c r="B21" s="17">
-        <v>74.04</v>
+        <v>313.5</v>
       </c>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.25">
@@ -1121,58 +1144,58 @@
         <v>4</v>
       </c>
       <c r="B5" s="6">
-        <v>46269.69564805555</v>
+        <v>46269.70988201389</v>
       </c>
     </row>
     <row r="6" ht="20" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A6" s="7" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="B6" s="7" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="C6" s="7" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="D6" s="7" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="E6" s="7" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="F6" s="7" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="G6" s="7" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="H6" s="7" t="s">
-        <v>56</v>
+        <v>68</v>
       </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A7" s="8" t="s">
+        <v>72</v>
+      </c>
+      <c r="B7" s="8" t="s">
         <v>70</v>
       </c>
-      <c r="B7" s="8" t="s">
-        <v>68</v>
-      </c>
       <c r="C7" s="19">
         <v>1</v>
       </c>
       <c r="D7" s="19">
-        <v>1</v>
-      </c>
-      <c r="E7" s="22">
+        <v>7</v>
+      </c>
+      <c r="E7" s="29">
         <v>400</v>
       </c>
-      <c r="F7" s="22">
+      <c r="F7" s="29">
         <v>0</v>
       </c>
-      <c r="G7" s="22">
+      <c r="G7" s="29">
         <f>C7*D7*E7+F7</f>
       </c>
-      <c r="H7" s="22">
+      <c r="H7" s="29">
         <f>G7*1.06</f>
       </c>
     </row>
@@ -1260,58 +1283,58 @@
         <v>4</v>
       </c>
       <c r="B5" s="6">
-        <v>46269.69564806713</v>
+        <v>46269.70988202546</v>
       </c>
     </row>
     <row r="6" ht="20" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A6" s="7" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="B6" s="7" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="C6" s="7" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="D6" s="7" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="E6" s="7" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="F6" s="7" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="G6" s="7" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="H6" s="7" t="s">
-        <v>56</v>
+        <v>68</v>
       </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A7" s="8" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="B7" s="8" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="C7" s="19">
         <v>1</v>
       </c>
-      <c r="D7" s="22">
+      <c r="D7" s="29">
         <v>500</v>
       </c>
       <c r="E7" s="8" t="s">
-        <v>77</v>
-      </c>
-      <c r="F7" s="22">
+        <v>79</v>
+      </c>
+      <c r="F7" s="29">
         <f>C7*D7</f>
       </c>
-      <c r="G7" s="22">
+      <c r="G7" s="29">
         <f>F7*0.065</f>
       </c>
-      <c r="H7" s="22">
+      <c r="H7" s="29">
         <f>F7+G7</f>
       </c>
     </row>
@@ -1397,52 +1420,52 @@
         <v>4</v>
       </c>
       <c r="B5" s="6">
-        <v>46269.69564806713</v>
+        <v>46269.70988202546</v>
       </c>
     </row>
     <row r="6" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" s="7" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="B6" s="7" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="C6" s="7" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="D6" s="7" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="E6" s="7" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="F6" s="7" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="G6" s="7" t="s">
-        <v>56</v>
+        <v>68</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" s="8" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="B7" s="8" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="C7" s="19">
         <v>1</v>
       </c>
       <c r="D7" s="19">
-        <v>1</v>
-      </c>
-      <c r="E7" s="22">
+        <v>7</v>
+      </c>
+      <c r="E7" s="29">
         <v>32</v>
       </c>
-      <c r="F7" s="22">
+      <c r="F7" s="29">
         <v>0</v>
       </c>
-      <c r="G7" s="22">
+      <c r="G7" s="29">
         <f>C7*D7*E7+F7</f>
       </c>
     </row>
@@ -1518,29 +1541,29 @@
         <v>4</v>
       </c>
       <c r="B5" s="6">
-        <v>46269.69564806713</v>
+        <v>46269.70988202546</v>
       </c>
     </row>
     <row r="6" ht="20" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" s="7" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="B6" s="7" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="C6" s="7" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="D6" s="7" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="E6" s="7" t="s">
-        <v>56</v>
+        <v>68</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" s="8" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="B7" s="19">
         <v>1</v>
@@ -1548,10 +1571,10 @@
       <c r="C7" s="19">
         <v>40</v>
       </c>
-      <c r="D7" s="22">
+      <c r="D7" s="29">
         <v>0.7</v>
       </c>
-      <c r="E7" s="22">
+      <c r="E7" s="29">
         <f>B7*C7*D7</f>
       </c>
     </row>
@@ -1628,40 +1651,40 @@
         <v>4</v>
       </c>
       <c r="B5" s="6">
-        <v>46269.69564806713</v>
+        <v>46269.70988202546</v>
       </c>
     </row>
     <row r="6" ht="20" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" s="7" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="B6" s="7" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="C6" s="7" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="D6" s="7" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="E6" s="7" t="s">
-        <v>56</v>
+        <v>68</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" s="8" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="B7" s="8" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="C7" s="19">
         <v>1</v>
       </c>
-      <c r="D7" s="22">
+      <c r="D7" s="29">
         <v>25</v>
       </c>
-      <c r="E7" s="22">
+      <c r="E7" s="29">
         <f>C7*D7</f>
       </c>
     </row>
@@ -1738,46 +1761,46 @@
         <v>4</v>
       </c>
       <c r="B5" s="6">
-        <v>46269.695648043984</v>
+        <v>46269.70988199074</v>
       </c>
     </row>
     <row r="6" ht="20" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" s="7" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="B6" s="7" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="C6" s="7" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="D6" s="7" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="E6" s="7" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="F6" s="7" t="s">
-        <v>51</v>
+        <v>95</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7" s="8" t="s">
         <v>30</v>
       </c>
-      <c r="B7" s="22">
+      <c r="B7" s="29">
         <v>52.5</v>
       </c>
-      <c r="C7" s="22">
+      <c r="C7" s="29">
         <v>91.02</v>
       </c>
-      <c r="D7" s="22">
+      <c r="D7" s="29">
         <v>122.2</v>
       </c>
-      <c r="E7" s="22">
+      <c r="E7" s="29">
         <v>153.39</v>
       </c>
-      <c r="F7" s="22">
+      <c r="F7" s="29">
         <v>140</v>
       </c>
     </row>
@@ -1785,19 +1808,19 @@
       <c r="A8" s="11" t="s">
         <v>34</v>
       </c>
-      <c r="B8" s="24">
+      <c r="B8" s="30">
         <v>58.84</v>
       </c>
-      <c r="C8" s="24">
+      <c r="C8" s="30">
         <v>111.22</v>
       </c>
-      <c r="D8" s="24">
+      <c r="D8" s="30">
         <v>156.31</v>
       </c>
-      <c r="E8" s="24">
+      <c r="E8" s="30">
         <v>201.4</v>
       </c>
-      <c r="F8" s="24">
+      <c r="F8" s="30">
         <v>140</v>
       </c>
     </row>
@@ -1805,39 +1828,39 @@
       <c r="A9" s="8" t="s">
         <v>36</v>
       </c>
-      <c r="B9" s="22">
+      <c r="B9" s="29">
         <v>49.1</v>
       </c>
-      <c r="C9" s="22">
+      <c r="C9" s="29">
         <v>112.62</v>
       </c>
-      <c r="D9" s="22">
+      <c r="D9" s="29">
         <v>159.07</v>
       </c>
-      <c r="E9" s="22">
+      <c r="E9" s="29">
         <v>205.52</v>
       </c>
-      <c r="F9" s="22">
+      <c r="F9" s="29">
         <v>130</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10" s="8" t="s">
-        <v>58</v>
-      </c>
-      <c r="B10" s="22">
+        <v>59</v>
+      </c>
+      <c r="B10" s="29">
         <v>45.6</v>
       </c>
-      <c r="C10" s="22">
+      <c r="C10" s="29">
         <v>108.38</v>
       </c>
-      <c r="D10" s="22">
+      <c r="D10" s="29">
         <v>152.78</v>
       </c>
-      <c r="E10" s="22">
+      <c r="E10" s="29">
         <v>197.19</v>
       </c>
-      <c r="F10" s="22">
+      <c r="F10" s="29">
         <v>130</v>
       </c>
     </row>
@@ -1906,7 +1929,7 @@
         <v>4</v>
       </c>
       <c r="B5" s="6">
-        <v>46269.69564805555</v>
+        <v>46269.70988201389</v>
       </c>
     </row>
     <row r="6" ht="20" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -2052,7 +2075,7 @@
         <v>4</v>
       </c>
       <c r="B5" s="6">
-        <v>46269.69564805555</v>
+        <v>46269.70988201389</v>
       </c>
     </row>
     <row r="6" ht="20" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -2077,13 +2100,13 @@
         <v>44</v>
       </c>
       <c r="B7" s="21">
-        <v>42</v>
+        <v>210</v>
       </c>
       <c r="C7" s="21">
-        <v>8</v>
+        <v>90</v>
       </c>
       <c r="D7" s="21">
-        <v>0</v>
+        <v>50</v>
       </c>
       <c r="E7" s="21">
         <f>B7+C7+D7</f>
@@ -2127,17 +2150,20 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr>
     <tabColor rgb="FF1F8A96"/>
-    <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:P9"/>
+  <dimension ref="A1:R21"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
-    <col min="1" max="1" width="32" customWidth="1"/>
-    <col min="2" max="6" width="12" customWidth="1"/>
-    <col min="7" max="16" width="14" customWidth="1"/>
+    <col min="1" max="1" width="28" customWidth="1"/>
+    <col min="2" max="2" width="14" customWidth="1"/>
+    <col min="3" max="3" width="26" customWidth="1"/>
+    <col min="4" max="5" width="14" customWidth="1"/>
+    <col min="6" max="10" width="12" customWidth="1"/>
+    <col min="11" max="11" width="14" customWidth="1"/>
+    <col min="12" max="18" width="7" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="22" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="1" ht="22" customHeight="1" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2156,13 +2182,15 @@
       <c r="N1" s="1"/>
       <c r="O1" s="1"/>
       <c r="P1" s="1"/>
+      <c r="Q1" s="1"/>
+      <c r="R1" s="1"/>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
         <v>2</v>
       </c>
@@ -2181,6 +2209,8 @@
       <c r="N3" s="3"/>
       <c r="O3" s="3"/>
       <c r="P3" s="3"/>
+      <c r="Q3" s="3"/>
+      <c r="R3" s="3"/>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A4" s="4" t="s">
@@ -2192,202 +2222,547 @@
         <v>4</v>
       </c>
       <c r="B5" s="6">
-        <v>46269.69564805555</v>
-      </c>
-    </row>
-    <row r="6" ht="20" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+        <v>46269.70988200232</v>
+      </c>
+    </row>
+    <row r="6" ht="20" customHeight="1" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A6" s="7" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="B6" s="7" t="s">
         <v>46</v>
       </c>
       <c r="C6" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="D6" s="7" t="s">
+        <v>47</v>
+      </c>
+      <c r="E6" s="7" t="s">
+        <v>48</v>
+      </c>
+      <c r="F6" s="7" t="s">
+        <v>49</v>
+      </c>
+      <c r="G6" s="7" t="s">
         <v>40</v>
       </c>
-      <c r="D6" s="7" t="s">
+      <c r="H6" s="7" t="s">
         <v>41</v>
       </c>
-      <c r="E6" s="7" t="s">
+      <c r="I6" s="7" t="s">
         <v>42</v>
       </c>
-      <c r="F6" s="7" t="s">
-        <v>47</v>
-      </c>
-      <c r="G6" s="7" t="s">
-        <v>48</v>
-      </c>
-      <c r="H6" s="7" t="s">
-        <v>49</v>
-      </c>
-      <c r="I6" s="7" t="s">
+      <c r="J6" s="7" t="s">
         <v>50</v>
       </c>
-      <c r="J6" s="7" t="s">
+      <c r="K6" s="7" t="s">
+        <v>12</v>
+      </c>
+      <c r="L6" s="22">
+        <v>46266</v>
+      </c>
+      <c r="M6" s="22">
+        <f>L6+1</f>
+      </c>
+      <c r="N6" s="22">
+        <f>M6+1</f>
+      </c>
+      <c r="O6" s="22">
+        <f>N6+1</f>
+      </c>
+      <c r="P6" s="22">
+        <f>O6+1</f>
+      </c>
+      <c r="Q6" s="22">
+        <f>P6+1</f>
+      </c>
+      <c r="R6" s="22">
+        <f>Q6+1</f>
+      </c>
+    </row>
+    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A7" s="23" t="s">
         <v>51</v>
       </c>
-      <c r="K6" s="7" t="s">
+      <c r="B7" s="24">
+        <f>G7+H7+I7</f>
+      </c>
+      <c r="C7" s="23" t="s">
+        <v>30</v>
+      </c>
+      <c r="D7" s="25">
+        <f>K7</f>
+      </c>
+      <c r="G7" s="24">
+        <f>B10</f>
+      </c>
+      <c r="H7" s="24">
+        <f>B11</f>
+      </c>
+      <c r="I7" s="24">
+        <f>B12</f>
+      </c>
+      <c r="J7" s="24">
+        <f>B13</f>
+      </c>
+      <c r="K7" s="25">
+        <f>D10+D11+D12</f>
+      </c>
+    </row>
+    <row r="8" spans="6:18" x14ac:dyDescent="0.25">
+      <c r="F8" s="26" t="s">
         <v>52</v>
       </c>
-      <c r="L6" s="7" t="s">
+      <c r="L8" s="27">
+        <v>1</v>
+      </c>
+      <c r="M8" s="27">
+        <v>1</v>
+      </c>
+      <c r="N8" s="27">
+        <v>1</v>
+      </c>
+      <c r="O8" s="27">
+        <v>1</v>
+      </c>
+      <c r="P8" s="27">
+        <v>1</v>
+      </c>
+      <c r="Q8" s="27">
+        <v>1</v>
+      </c>
+      <c r="R8" s="27">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A9" s="26" t="s">
         <v>53</v>
       </c>
-      <c r="M6" s="7" t="s">
+      <c r="F9" s="26" t="s">
         <v>54</v>
       </c>
-      <c r="N6" s="7" t="s">
+      <c r="L9" s="28">
+        <v>10</v>
+      </c>
+      <c r="M9" s="28">
+        <v>10</v>
+      </c>
+      <c r="N9" s="28">
+        <v>10</v>
+      </c>
+      <c r="O9" s="28">
+        <v>10</v>
+      </c>
+      <c r="P9" s="28">
+        <v>10</v>
+      </c>
+      <c r="Q9" s="28">
+        <v>10</v>
+      </c>
+      <c r="R9" s="28">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="10" spans="2:18" x14ac:dyDescent="0.25">
+      <c r="B10" s="21">
+        <f>SUM(L10:R10)</f>
+      </c>
+      <c r="D10" s="29">
+        <f>B10*E10</f>
+      </c>
+      <c r="E10" s="29">
+        <f>'Rate Tables'!C7</f>
+      </c>
+      <c r="F10" s="8" t="s">
         <v>55</v>
       </c>
-      <c r="O6" s="7" t="s">
+      <c r="L10" s="21">
+        <f>IF(L$6="","",IF(WEEKDAY(L$6,1)=1,0,MIN(10,L9)*L8))</f>
+      </c>
+      <c r="M10" s="21">
+        <f>IF(M$6="","",IF(WEEKDAY(M$6,1)=1,0,MIN(10,M9)*M8))</f>
+      </c>
+      <c r="N10" s="21">
+        <f>IF(N$6="","",IF(WEEKDAY(N$6,1)=1,0,MIN(10,N9)*N8))</f>
+      </c>
+      <c r="O10" s="21">
+        <f>IF(O$6="","",IF(WEEKDAY(O$6,1)=1,0,MIN(10,O9)*O8))</f>
+      </c>
+      <c r="P10" s="21">
+        <f>IF(P$6="","",IF(WEEKDAY(P$6,1)=1,0,MIN(10,P9)*P8))</f>
+      </c>
+      <c r="Q10" s="21">
+        <f>IF(Q$6="","",IF(WEEKDAY(Q$6,1)=1,0,MIN(10,Q9)*Q8))</f>
+      </c>
+      <c r="R10" s="21">
+        <f>IF(R$6="","",IF(WEEKDAY(R$6,1)=1,0,MIN(10,R9)*R8))</f>
+      </c>
+    </row>
+    <row r="11" spans="2:18" x14ac:dyDescent="0.25">
+      <c r="B11" s="21">
+        <f>SUM(L11:R11)</f>
+      </c>
+      <c r="D11" s="29">
+        <f>B11*E11</f>
+      </c>
+      <c r="E11" s="29">
+        <f>'Rate Tables'!D7</f>
+      </c>
+      <c r="F11" s="8" t="s">
         <v>56</v>
       </c>
-      <c r="P6" s="7" t="s">
+      <c r="L11" s="21">
+        <f>IF(L$6="","",IF(WEEKDAY(L$6,1)=1,0,MAX(0,L9-10)*L8))</f>
+      </c>
+      <c r="M11" s="21">
+        <f>IF(M$6="","",IF(WEEKDAY(M$6,1)=1,0,MAX(0,M9-10)*M8))</f>
+      </c>
+      <c r="N11" s="21">
+        <f>IF(N$6="","",IF(WEEKDAY(N$6,1)=1,0,MAX(0,N9-10)*N8))</f>
+      </c>
+      <c r="O11" s="21">
+        <f>IF(O$6="","",IF(WEEKDAY(O$6,1)=1,0,MAX(0,O9-10)*O8))</f>
+      </c>
+      <c r="P11" s="21">
+        <f>IF(P$6="","",IF(WEEKDAY(P$6,1)=1,0,MAX(0,P9-10)*P8))</f>
+      </c>
+      <c r="Q11" s="21">
+        <f>IF(Q$6="","",IF(WEEKDAY(Q$6,1)=1,0,MAX(0,Q9-10)*Q8))</f>
+      </c>
+      <c r="R11" s="21">
+        <f>IF(R$6="","",IF(WEEKDAY(R$6,1)=1,0,MAX(0,R9-10)*R8))</f>
+      </c>
+    </row>
+    <row r="12" spans="2:18" x14ac:dyDescent="0.25">
+      <c r="B12" s="21">
+        <f>SUM(L12:R12)</f>
+      </c>
+      <c r="D12" s="29">
+        <f>B12*E12</f>
+      </c>
+      <c r="E12" s="29">
+        <f>'Rate Tables'!E7</f>
+      </c>
+      <c r="F12" s="8" t="s">
         <v>57</v>
       </c>
-    </row>
-    <row r="7" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A7" s="8" t="s">
-        <v>30</v>
-      </c>
-      <c r="B7" s="19">
-        <v>1</v>
-      </c>
-      <c r="C7" s="21">
+      <c r="L12" s="21">
+        <f>IF(L$6="","",IF(WEEKDAY(L$6,1)=1,L9*L8,0))</f>
+      </c>
+      <c r="M12" s="21">
+        <f>IF(M$6="","",IF(WEEKDAY(M$6,1)=1,M9*M8,0))</f>
+      </c>
+      <c r="N12" s="21">
+        <f>IF(N$6="","",IF(WEEKDAY(N$6,1)=1,N9*N8,0))</f>
+      </c>
+      <c r="O12" s="21">
+        <f>IF(O$6="","",IF(WEEKDAY(O$6,1)=1,O9*O8,0))</f>
+      </c>
+      <c r="P12" s="21">
+        <f>IF(P$6="","",IF(WEEKDAY(P$6,1)=1,P9*P8,0))</f>
+      </c>
+      <c r="Q12" s="21">
+        <f>IF(Q$6="","",IF(WEEKDAY(Q$6,1)=1,Q9*Q8,0))</f>
+      </c>
+      <c r="R12" s="21">
+        <f>IF(R$6="","",IF(WEEKDAY(R$6,1)=1,R9*R8,0))</f>
+      </c>
+    </row>
+    <row r="13" spans="2:18" x14ac:dyDescent="0.25">
+      <c r="B13" s="21">
+        <f>SUM(L13:R13)</f>
+      </c>
+      <c r="D13" s="29">
+        <f>B13*E13</f>
+      </c>
+      <c r="E13" s="29">
+        <v>140</v>
+      </c>
+      <c r="F13" s="8" t="s">
+        <v>58</v>
+      </c>
+      <c r="L13" s="19">
+        <v>1</v>
+      </c>
+      <c r="M13" s="19">
+        <v>1</v>
+      </c>
+      <c r="N13" s="19">
+        <v>1</v>
+      </c>
+      <c r="O13" s="19">
+        <v>1</v>
+      </c>
+      <c r="P13" s="19">
+        <v>1</v>
+      </c>
+      <c r="Q13" s="19">
+        <v>1</v>
+      </c>
+      <c r="R13" s="19">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="14" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A14" s="23" t="s">
+        <v>51</v>
+      </c>
+      <c r="B14" s="24">
+        <f>G14+H14+I14</f>
+      </c>
+      <c r="C14" s="23" t="s">
+        <v>34</v>
+      </c>
+      <c r="D14" s="25">
+        <f>K14</f>
+      </c>
+      <c r="G14" s="24">
+        <f>B17</f>
+      </c>
+      <c r="H14" s="24">
+        <f>B18</f>
+      </c>
+      <c r="I14" s="24">
+        <f>B19</f>
+      </c>
+      <c r="J14" s="24">
+        <f>B20</f>
+      </c>
+      <c r="K14" s="25">
+        <f>D17+D18+D19</f>
+      </c>
+    </row>
+    <row r="15" spans="6:18" x14ac:dyDescent="0.25">
+      <c r="F15" s="26" t="s">
+        <v>52</v>
+      </c>
+      <c r="L15" s="27">
+        <v>1</v>
+      </c>
+      <c r="M15" s="27">
+        <v>1</v>
+      </c>
+      <c r="N15" s="27">
+        <v>1</v>
+      </c>
+      <c r="O15" s="27">
+        <v>1</v>
+      </c>
+      <c r="P15" s="27">
+        <v>1</v>
+      </c>
+      <c r="Q15" s="27">
+        <v>1</v>
+      </c>
+      <c r="R15" s="27">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="16" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A16" s="26" t="s">
+        <v>53</v>
+      </c>
+      <c r="F16" s="26" t="s">
+        <v>54</v>
+      </c>
+      <c r="L16" s="28">
         <v>10</v>
       </c>
-      <c r="D7" s="21">
-        <v>0</v>
-      </c>
-      <c r="E7" s="21">
-        <v>0</v>
-      </c>
-      <c r="F7" s="21">
-        <v>1</v>
-      </c>
-      <c r="G7" s="22">
-        <f>'Rate Tables'!C7</f>
-      </c>
-      <c r="H7" s="22">
-        <f>'Rate Tables'!D7</f>
-      </c>
-      <c r="I7" s="22">
-        <f>'Rate Tables'!E7</f>
-      </c>
-      <c r="J7" s="22">
+      <c r="M16" s="28">
+        <v>10</v>
+      </c>
+      <c r="N16" s="28">
+        <v>10</v>
+      </c>
+      <c r="O16" s="28">
+        <v>10</v>
+      </c>
+      <c r="P16" s="28">
+        <v>10</v>
+      </c>
+      <c r="Q16" s="28">
+        <v>10</v>
+      </c>
+      <c r="R16" s="28">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="17" spans="2:18" x14ac:dyDescent="0.25">
+      <c r="B17" s="21">
+        <f>SUM(L17:R17)</f>
+      </c>
+      <c r="D17" s="29">
+        <f>B17*E17</f>
+      </c>
+      <c r="E17" s="29">
+        <f>'Rate Tables'!C8</f>
+      </c>
+      <c r="F17" s="8" t="s">
+        <v>55</v>
+      </c>
+      <c r="L17" s="21">
+        <f>IF(L$6="","",IF(OR(WEEKDAY(L$6,1)=1,WEEKDAY(L$6,1)=7),0,MIN(8,L16)*L15))</f>
+      </c>
+      <c r="M17" s="21">
+        <f>IF(M$6="","",IF(OR(WEEKDAY(M$6,1)=1,WEEKDAY(M$6,1)=7),0,MIN(8,M16)*M15))</f>
+      </c>
+      <c r="N17" s="21">
+        <f>IF(N$6="","",IF(OR(WEEKDAY(N$6,1)=1,WEEKDAY(N$6,1)=7),0,MIN(8,N16)*N15))</f>
+      </c>
+      <c r="O17" s="21">
+        <f>IF(O$6="","",IF(OR(WEEKDAY(O$6,1)=1,WEEKDAY(O$6,1)=7),0,MIN(8,O16)*O15))</f>
+      </c>
+      <c r="P17" s="21">
+        <f>IF(P$6="","",IF(OR(WEEKDAY(P$6,1)=1,WEEKDAY(P$6,1)=7),0,MIN(8,P16)*P15))</f>
+      </c>
+      <c r="Q17" s="21">
+        <f>IF(Q$6="","",IF(OR(WEEKDAY(Q$6,1)=1,WEEKDAY(Q$6,1)=7),0,MIN(8,Q16)*Q15))</f>
+      </c>
+      <c r="R17" s="21">
+        <f>IF(R$6="","",IF(OR(WEEKDAY(R$6,1)=1,WEEKDAY(R$6,1)=7),0,MIN(8,R16)*R15))</f>
+      </c>
+    </row>
+    <row r="18" spans="2:18" x14ac:dyDescent="0.25">
+      <c r="B18" s="21">
+        <f>SUM(L18:R18)</f>
+      </c>
+      <c r="D18" s="29">
+        <f>B18*E18</f>
+      </c>
+      <c r="E18" s="29">
+        <f>'Rate Tables'!D8</f>
+      </c>
+      <c r="F18" s="8" t="s">
+        <v>56</v>
+      </c>
+      <c r="L18" s="21">
+        <f>IF(L$6="","",IF(WEEKDAY(L$6,1)=1,0,IF(WEEKDAY(L$6,1)=7,L16*L15,MAX(0,L16-8)*L15)))</f>
+      </c>
+      <c r="M18" s="21">
+        <f>IF(M$6="","",IF(WEEKDAY(M$6,1)=1,0,IF(WEEKDAY(M$6,1)=7,M16*M15,MAX(0,M16-8)*M15)))</f>
+      </c>
+      <c r="N18" s="21">
+        <f>IF(N$6="","",IF(WEEKDAY(N$6,1)=1,0,IF(WEEKDAY(N$6,1)=7,N16*N15,MAX(0,N16-8)*N15)))</f>
+      </c>
+      <c r="O18" s="21">
+        <f>IF(O$6="","",IF(WEEKDAY(O$6,1)=1,0,IF(WEEKDAY(O$6,1)=7,O16*O15,MAX(0,O16-8)*O15)))</f>
+      </c>
+      <c r="P18" s="21">
+        <f>IF(P$6="","",IF(WEEKDAY(P$6,1)=1,0,IF(WEEKDAY(P$6,1)=7,P16*P15,MAX(0,P16-8)*P15)))</f>
+      </c>
+      <c r="Q18" s="21">
+        <f>IF(Q$6="","",IF(WEEKDAY(Q$6,1)=1,0,IF(WEEKDAY(Q$6,1)=7,Q16*Q15,MAX(0,Q16-8)*Q15)))</f>
+      </c>
+      <c r="R18" s="21">
+        <f>IF(R$6="","",IF(WEEKDAY(R$6,1)=1,0,IF(WEEKDAY(R$6,1)=7,R16*R15,MAX(0,R16-8)*R15)))</f>
+      </c>
+    </row>
+    <row r="19" spans="2:18" x14ac:dyDescent="0.25">
+      <c r="B19" s="21">
+        <f>SUM(L19:R19)</f>
+      </c>
+      <c r="D19" s="29">
+        <f>B19*E19</f>
+      </c>
+      <c r="E19" s="29">
+        <f>'Rate Tables'!E8</f>
+      </c>
+      <c r="F19" s="8" t="s">
+        <v>57</v>
+      </c>
+      <c r="L19" s="21">
+        <f>IF(L$6="","",IF(WEEKDAY(L$6,1)=1,L16*L15,0))</f>
+      </c>
+      <c r="M19" s="21">
+        <f>IF(M$6="","",IF(WEEKDAY(M$6,1)=1,M16*M15,0))</f>
+      </c>
+      <c r="N19" s="21">
+        <f>IF(N$6="","",IF(WEEKDAY(N$6,1)=1,N16*N15,0))</f>
+      </c>
+      <c r="O19" s="21">
+        <f>IF(O$6="","",IF(WEEKDAY(O$6,1)=1,O16*O15,0))</f>
+      </c>
+      <c r="P19" s="21">
+        <f>IF(P$6="","",IF(WEEKDAY(P$6,1)=1,P16*P15,0))</f>
+      </c>
+      <c r="Q19" s="21">
+        <f>IF(Q$6="","",IF(WEEKDAY(Q$6,1)=1,Q16*Q15,0))</f>
+      </c>
+      <c r="R19" s="21">
+        <f>IF(R$6="","",IF(WEEKDAY(R$6,1)=1,R16*R15,0))</f>
+      </c>
+    </row>
+    <row r="20" spans="2:18" x14ac:dyDescent="0.25">
+      <c r="B20" s="21">
+        <f>SUM(L20:R20)</f>
+      </c>
+      <c r="D20" s="29">
+        <f>B20*E20</f>
+      </c>
+      <c r="E20" s="29">
         <v>140</v>
       </c>
-      <c r="K7" s="22">
-        <f>C7*G7</f>
-      </c>
-      <c r="L7" s="22">
-        <f>D7*H7</f>
-      </c>
-      <c r="M7" s="22">
-        <f>E7*I7</f>
-      </c>
-      <c r="N7" s="22">
-        <f>F7*J7</f>
-      </c>
-      <c r="O7" s="22">
-        <f>K7+L7+M7</f>
-      </c>
-      <c r="P7" s="21">
-        <f>C7+D7+E7</f>
-      </c>
-    </row>
-    <row r="8" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A8" s="11" t="s">
-        <v>34</v>
-      </c>
-      <c r="B8" s="20">
-        <v>1</v>
-      </c>
-      <c r="C8" s="23">
-        <v>8</v>
-      </c>
-      <c r="D8" s="23">
-        <v>2</v>
-      </c>
-      <c r="E8" s="23">
-        <v>0</v>
-      </c>
-      <c r="F8" s="23">
-        <v>1</v>
-      </c>
-      <c r="G8" s="24">
-        <f>'Rate Tables'!C8</f>
-      </c>
-      <c r="H8" s="24">
-        <f>'Rate Tables'!D8</f>
-      </c>
-      <c r="I8" s="24">
-        <f>'Rate Tables'!E8</f>
-      </c>
-      <c r="J8" s="24">
-        <v>140</v>
-      </c>
-      <c r="K8" s="24">
-        <f>C8*G8</f>
-      </c>
-      <c r="L8" s="24">
-        <f>D8*H8</f>
-      </c>
-      <c r="M8" s="24">
-        <f>E8*I8</f>
-      </c>
-      <c r="N8" s="24">
-        <f>F8*J8</f>
-      </c>
-      <c r="O8" s="24">
-        <f>K8+L8+M8</f>
-      </c>
-      <c r="P8" s="23">
-        <f>C8+D8+E8</f>
-      </c>
-    </row>
-    <row r="9" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A9" s="14" t="s">
+      <c r="F20" s="8" t="s">
+        <v>58</v>
+      </c>
+      <c r="L20" s="19">
+        <v>1</v>
+      </c>
+      <c r="M20" s="19">
+        <v>1</v>
+      </c>
+      <c r="N20" s="19">
+        <v>1</v>
+      </c>
+      <c r="O20" s="19">
+        <v>1</v>
+      </c>
+      <c r="P20" s="19">
+        <v>1</v>
+      </c>
+      <c r="Q20" s="19">
+        <v>1</v>
+      </c>
+      <c r="R20" s="19">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="21" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A21" s="14" t="s">
         <v>45</v>
       </c>
-      <c r="C9" s="15">
-        <f>SUM(C7:C8)</f>
-      </c>
-      <c r="D9" s="15">
-        <f>SUM(D7:D8)</f>
-      </c>
-      <c r="E9" s="15">
-        <f>SUM(E7:E8)</f>
-      </c>
-      <c r="F9" s="15">
-        <f>SUM(F7:F8)</f>
-      </c>
-      <c r="K9" s="18">
-        <f>SUM(K7:K8)</f>
-      </c>
-      <c r="L9" s="18">
-        <f>SUM(L7:L8)</f>
-      </c>
-      <c r="M9" s="18">
-        <f>SUM(M7:M8)</f>
-      </c>
-      <c r="N9" s="18">
-        <f>SUM(N7:N8)</f>
-      </c>
-      <c r="O9" s="18">
-        <f>SUM(O7:O8)</f>
-      </c>
-      <c r="P9" s="15">
-        <f>SUM(P7:P8)</f>
+      <c r="B21" s="15">
+        <f>SUM(B7,B14)</f>
+      </c>
+      <c r="D21" s="18">
+        <f>SUM(D13,D20)</f>
+      </c>
+      <c r="G21" s="15">
+        <f>SUM(G7,G14)</f>
+      </c>
+      <c r="H21" s="15">
+        <f>SUM(H7,H14)</f>
+      </c>
+      <c r="I21" s="15">
+        <f>SUM(I7,I14)</f>
+      </c>
+      <c r="J21" s="15">
+        <f>SUM(J7,J14)</f>
+      </c>
+      <c r="K21" s="18">
+        <f>SUM(K7,K14)</f>
       </c>
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A1:P1"/>
-    <mergeCell ref="A3:P3"/>
+    <mergeCell ref="A1:R1"/>
+    <mergeCell ref="A3:R3"/>
   </mergeCells>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.4" right="0.4" top="0.65" bottom="0.65" header="0.28" footer="0.28"/>
-  <pageSetup orientation="landscape" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="20"/>
+  <pageSetup orientation="landscape" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100"/>
   <headerFooter>
     <oddHeader>&amp;L&amp;B HIT SQUAD / PROJECT CONTROLS &amp;C Staff &amp;R Confidential</oddHeader>
     <oddFooter>&amp;L Produced by Hit Squad Project Controls &amp;C &amp;D &amp;R Page &amp;P of &amp;N</oddFooter>
@@ -2401,17 +2776,20 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr>
     <tabColor rgb="FF1F8A96"/>
-    <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:P8"/>
+  <dimension ref="A1:R14"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
-    <col min="1" max="1" width="32" customWidth="1"/>
-    <col min="2" max="6" width="12" customWidth="1"/>
-    <col min="7" max="16" width="14" customWidth="1"/>
+    <col min="1" max="1" width="28" customWidth="1"/>
+    <col min="2" max="2" width="14" customWidth="1"/>
+    <col min="3" max="3" width="26" customWidth="1"/>
+    <col min="4" max="5" width="14" customWidth="1"/>
+    <col min="6" max="10" width="12" customWidth="1"/>
+    <col min="11" max="11" width="14" customWidth="1"/>
+    <col min="12" max="18" width="7" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="22" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="1" ht="22" customHeight="1" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2430,13 +2808,15 @@
       <c r="N1" s="1"/>
       <c r="O1" s="1"/>
       <c r="P1" s="1"/>
+      <c r="Q1" s="1"/>
+      <c r="R1" s="1"/>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
         <v>2</v>
       </c>
@@ -2455,6 +2835,8 @@
       <c r="N3" s="3"/>
       <c r="O3" s="3"/>
       <c r="P3" s="3"/>
+      <c r="Q3" s="3"/>
+      <c r="R3" s="3"/>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A4" s="4" t="s">
@@ -2466,152 +2848,323 @@
         <v>4</v>
       </c>
       <c r="B5" s="6">
-        <v>46269.69564805555</v>
-      </c>
-    </row>
-    <row r="6" ht="20" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+        <v>46269.70988200232</v>
+      </c>
+    </row>
+    <row r="6" ht="20" customHeight="1" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A6" s="7" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="B6" s="7" t="s">
         <v>46</v>
       </c>
       <c r="C6" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="D6" s="7" t="s">
+        <v>47</v>
+      </c>
+      <c r="E6" s="7" t="s">
+        <v>48</v>
+      </c>
+      <c r="F6" s="7" t="s">
+        <v>49</v>
+      </c>
+      <c r="G6" s="7" t="s">
         <v>40</v>
       </c>
-      <c r="D6" s="7" t="s">
+      <c r="H6" s="7" t="s">
         <v>41</v>
       </c>
-      <c r="E6" s="7" t="s">
+      <c r="I6" s="7" t="s">
         <v>42</v>
       </c>
-      <c r="F6" s="7" t="s">
-        <v>47</v>
-      </c>
-      <c r="G6" s="7" t="s">
-        <v>48</v>
-      </c>
-      <c r="H6" s="7" t="s">
-        <v>49</v>
-      </c>
-      <c r="I6" s="7" t="s">
+      <c r="J6" s="7" t="s">
         <v>50</v>
       </c>
-      <c r="J6" s="7" t="s">
+      <c r="K6" s="7" t="s">
+        <v>12</v>
+      </c>
+      <c r="L6" s="22">
+        <v>46266</v>
+      </c>
+      <c r="M6" s="22">
+        <f>L6+1</f>
+      </c>
+      <c r="N6" s="22">
+        <f>M6+1</f>
+      </c>
+      <c r="O6" s="22">
+        <f>N6+1</f>
+      </c>
+      <c r="P6" s="22">
+        <f>O6+1</f>
+      </c>
+      <c r="Q6" s="22">
+        <f>P6+1</f>
+      </c>
+      <c r="R6" s="22">
+        <f>Q6+1</f>
+      </c>
+    </row>
+    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A7" s="23" t="s">
         <v>51</v>
       </c>
-      <c r="K6" s="7" t="s">
+      <c r="B7" s="24">
+        <f>G7+H7+I7</f>
+      </c>
+      <c r="C7" s="23" t="s">
+        <v>36</v>
+      </c>
+      <c r="D7" s="25">
+        <f>K7</f>
+      </c>
+      <c r="G7" s="24">
+        <f>B10</f>
+      </c>
+      <c r="H7" s="24">
+        <f>B11</f>
+      </c>
+      <c r="I7" s="24">
+        <f>B12</f>
+      </c>
+      <c r="J7" s="24">
+        <f>B13</f>
+      </c>
+      <c r="K7" s="25">
+        <f>D10+D11+D12</f>
+      </c>
+    </row>
+    <row r="8" spans="6:18" x14ac:dyDescent="0.25">
+      <c r="F8" s="26" t="s">
         <v>52</v>
       </c>
-      <c r="L6" s="7" t="s">
+      <c r="L8" s="27">
+        <v>1</v>
+      </c>
+      <c r="M8" s="27">
+        <v>1</v>
+      </c>
+      <c r="N8" s="27">
+        <v>1</v>
+      </c>
+      <c r="O8" s="27">
+        <v>1</v>
+      </c>
+      <c r="P8" s="27">
+        <v>1</v>
+      </c>
+      <c r="Q8" s="27">
+        <v>1</v>
+      </c>
+      <c r="R8" s="27">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A9" s="26" t="s">
         <v>53</v>
       </c>
-      <c r="M6" s="7" t="s">
+      <c r="F9" s="26" t="s">
         <v>54</v>
       </c>
-      <c r="N6" s="7" t="s">
+      <c r="L9" s="28">
+        <v>10</v>
+      </c>
+      <c r="M9" s="28">
+        <v>10</v>
+      </c>
+      <c r="N9" s="28">
+        <v>10</v>
+      </c>
+      <c r="O9" s="28">
+        <v>10</v>
+      </c>
+      <c r="P9" s="28">
+        <v>10</v>
+      </c>
+      <c r="Q9" s="28">
+        <v>10</v>
+      </c>
+      <c r="R9" s="28">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="10" spans="2:18" x14ac:dyDescent="0.25">
+      <c r="B10" s="21">
+        <f>SUM(L10:R10)</f>
+      </c>
+      <c r="D10" s="29">
+        <f>B10*E10</f>
+      </c>
+      <c r="E10" s="29">
+        <f>'Rate Tables'!C9</f>
+      </c>
+      <c r="F10" s="8" t="s">
         <v>55</v>
       </c>
-      <c r="O6" s="7" t="s">
+      <c r="L10" s="21">
+        <f>IF(L$6="","",IF(OR(WEEKDAY(L$6,1)=1,WEEKDAY(L$6,1)=7),0,MIN(8,L9)*L8))</f>
+      </c>
+      <c r="M10" s="21">
+        <f>IF(M$6="","",IF(OR(WEEKDAY(M$6,1)=1,WEEKDAY(M$6,1)=7),0,MIN(8,M9)*M8))</f>
+      </c>
+      <c r="N10" s="21">
+        <f>IF(N$6="","",IF(OR(WEEKDAY(N$6,1)=1,WEEKDAY(N$6,1)=7),0,MIN(8,N9)*N8))</f>
+      </c>
+      <c r="O10" s="21">
+        <f>IF(O$6="","",IF(OR(WEEKDAY(O$6,1)=1,WEEKDAY(O$6,1)=7),0,MIN(8,O9)*O8))</f>
+      </c>
+      <c r="P10" s="21">
+        <f>IF(P$6="","",IF(OR(WEEKDAY(P$6,1)=1,WEEKDAY(P$6,1)=7),0,MIN(8,P9)*P8))</f>
+      </c>
+      <c r="Q10" s="21">
+        <f>IF(Q$6="","",IF(OR(WEEKDAY(Q$6,1)=1,WEEKDAY(Q$6,1)=7),0,MIN(8,Q9)*Q8))</f>
+      </c>
+      <c r="R10" s="21">
+        <f>IF(R$6="","",IF(OR(WEEKDAY(R$6,1)=1,WEEKDAY(R$6,1)=7),0,MIN(8,R9)*R8))</f>
+      </c>
+    </row>
+    <row r="11" spans="2:18" x14ac:dyDescent="0.25">
+      <c r="B11" s="21">
+        <f>SUM(L11:R11)</f>
+      </c>
+      <c r="D11" s="29">
+        <f>B11*E11</f>
+      </c>
+      <c r="E11" s="29">
+        <f>'Rate Tables'!D9</f>
+      </c>
+      <c r="F11" s="8" t="s">
         <v>56</v>
       </c>
-      <c r="P6" s="7" t="s">
+      <c r="L11" s="21">
+        <f>IF(L$6="","",IF(WEEKDAY(L$6,1)=1,0,IF(WEEKDAY(L$6,1)=7,L9*L8,MAX(0,L9-8)*L8)))</f>
+      </c>
+      <c r="M11" s="21">
+        <f>IF(M$6="","",IF(WEEKDAY(M$6,1)=1,0,IF(WEEKDAY(M$6,1)=7,M9*M8,MAX(0,M9-8)*M8)))</f>
+      </c>
+      <c r="N11" s="21">
+        <f>IF(N$6="","",IF(WEEKDAY(N$6,1)=1,0,IF(WEEKDAY(N$6,1)=7,N9*N8,MAX(0,N9-8)*N8)))</f>
+      </c>
+      <c r="O11" s="21">
+        <f>IF(O$6="","",IF(WEEKDAY(O$6,1)=1,0,IF(WEEKDAY(O$6,1)=7,O9*O8,MAX(0,O9-8)*O8)))</f>
+      </c>
+      <c r="P11" s="21">
+        <f>IF(P$6="","",IF(WEEKDAY(P$6,1)=1,0,IF(WEEKDAY(P$6,1)=7,P9*P8,MAX(0,P9-8)*P8)))</f>
+      </c>
+      <c r="Q11" s="21">
+        <f>IF(Q$6="","",IF(WEEKDAY(Q$6,1)=1,0,IF(WEEKDAY(Q$6,1)=7,Q9*Q8,MAX(0,Q9-8)*Q8)))</f>
+      </c>
+      <c r="R11" s="21">
+        <f>IF(R$6="","",IF(WEEKDAY(R$6,1)=1,0,IF(WEEKDAY(R$6,1)=7,R9*R8,MAX(0,R9-8)*R8)))</f>
+      </c>
+    </row>
+    <row r="12" spans="2:18" x14ac:dyDescent="0.25">
+      <c r="B12" s="21">
+        <f>SUM(L12:R12)</f>
+      </c>
+      <c r="D12" s="29">
+        <f>B12*E12</f>
+      </c>
+      <c r="E12" s="29">
+        <f>'Rate Tables'!E9</f>
+      </c>
+      <c r="F12" s="8" t="s">
         <v>57</v>
       </c>
-    </row>
-    <row r="7" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A7" s="8" t="s">
-        <v>36</v>
-      </c>
-      <c r="B7" s="19">
-        <v>1</v>
-      </c>
-      <c r="C7" s="21">
-        <v>8</v>
-      </c>
-      <c r="D7" s="21">
-        <v>2</v>
-      </c>
-      <c r="E7" s="21">
-        <v>0</v>
-      </c>
-      <c r="F7" s="21">
-        <v>1</v>
-      </c>
-      <c r="G7" s="22">
-        <f>'Rate Tables'!C9</f>
-      </c>
-      <c r="H7" s="22">
-        <f>'Rate Tables'!D9</f>
-      </c>
-      <c r="I7" s="22">
-        <f>'Rate Tables'!E9</f>
-      </c>
-      <c r="J7" s="22">
+      <c r="L12" s="21">
+        <f>IF(L$6="","",IF(WEEKDAY(L$6,1)=1,L9*L8,0))</f>
+      </c>
+      <c r="M12" s="21">
+        <f>IF(M$6="","",IF(WEEKDAY(M$6,1)=1,M9*M8,0))</f>
+      </c>
+      <c r="N12" s="21">
+        <f>IF(N$6="","",IF(WEEKDAY(N$6,1)=1,N9*N8,0))</f>
+      </c>
+      <c r="O12" s="21">
+        <f>IF(O$6="","",IF(WEEKDAY(O$6,1)=1,O9*O8,0))</f>
+      </c>
+      <c r="P12" s="21">
+        <f>IF(P$6="","",IF(WEEKDAY(P$6,1)=1,P9*P8,0))</f>
+      </c>
+      <c r="Q12" s="21">
+        <f>IF(Q$6="","",IF(WEEKDAY(Q$6,1)=1,Q9*Q8,0))</f>
+      </c>
+      <c r="R12" s="21">
+        <f>IF(R$6="","",IF(WEEKDAY(R$6,1)=1,R9*R8,0))</f>
+      </c>
+    </row>
+    <row r="13" spans="2:18" x14ac:dyDescent="0.25">
+      <c r="B13" s="21">
+        <f>SUM(L13:R13)</f>
+      </c>
+      <c r="D13" s="29">
+        <f>B13*E13</f>
+      </c>
+      <c r="E13" s="29">
         <v>130</v>
       </c>
-      <c r="K7" s="22">
-        <f>C7*G7</f>
-      </c>
-      <c r="L7" s="22">
-        <f>D7*H7</f>
-      </c>
-      <c r="M7" s="22">
-        <f>E7*I7</f>
-      </c>
-      <c r="N7" s="22">
-        <f>F7*J7</f>
-      </c>
-      <c r="O7" s="22">
-        <f>K7+L7+M7</f>
-      </c>
-      <c r="P7" s="21">
-        <f>C7+D7+E7</f>
-      </c>
-    </row>
-    <row r="8" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A8" s="14" t="s">
+      <c r="F13" s="8" t="s">
+        <v>58</v>
+      </c>
+      <c r="L13" s="19">
+        <v>1</v>
+      </c>
+      <c r="M13" s="19">
+        <v>1</v>
+      </c>
+      <c r="N13" s="19">
+        <v>1</v>
+      </c>
+      <c r="O13" s="19">
+        <v>1</v>
+      </c>
+      <c r="P13" s="19">
+        <v>1</v>
+      </c>
+      <c r="Q13" s="19">
+        <v>1</v>
+      </c>
+      <c r="R13" s="19">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="14" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A14" s="14" t="s">
         <v>45</v>
       </c>
-      <c r="C8" s="15">
-        <f>SUM(C7:C7)</f>
-      </c>
-      <c r="D8" s="15">
-        <f>SUM(D7:D7)</f>
-      </c>
-      <c r="E8" s="15">
-        <f>SUM(E7:E7)</f>
-      </c>
-      <c r="F8" s="15">
-        <f>SUM(F7:F7)</f>
-      </c>
-      <c r="K8" s="18">
-        <f>SUM(K7:K7)</f>
-      </c>
-      <c r="L8" s="18">
-        <f>SUM(L7:L7)</f>
-      </c>
-      <c r="M8" s="18">
-        <f>SUM(M7:M7)</f>
-      </c>
-      <c r="N8" s="18">
-        <f>SUM(N7:N7)</f>
-      </c>
-      <c r="O8" s="18">
-        <f>SUM(O7:O7)</f>
-      </c>
-      <c r="P8" s="15">
-        <f>SUM(P7:P7)</f>
+      <c r="B14" s="15">
+        <f>SUM(B7)</f>
+      </c>
+      <c r="D14" s="18">
+        <f>SUM(D13)</f>
+      </c>
+      <c r="G14" s="15">
+        <f>SUM(G7)</f>
+      </c>
+      <c r="H14" s="15">
+        <f>SUM(H7)</f>
+      </c>
+      <c r="I14" s="15">
+        <f>SUM(I7)</f>
+      </c>
+      <c r="J14" s="15">
+        <f>SUM(J7)</f>
+      </c>
+      <c r="K14" s="18">
+        <f>SUM(K7)</f>
       </c>
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A1:P1"/>
-    <mergeCell ref="A3:P3"/>
+    <mergeCell ref="A1:R1"/>
+    <mergeCell ref="A3:R3"/>
   </mergeCells>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.4" right="0.4" top="0.65" bottom="0.65" header="0.28" footer="0.28"/>
-  <pageSetup orientation="landscape" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="20"/>
+  <pageSetup orientation="landscape" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100"/>
   <headerFooter>
     <oddHeader>&amp;L&amp;B HIT SQUAD / PROJECT CONTROLS &amp;C Foremen &amp;R Confidential</oddHeader>
     <oddFooter>&amp;L Produced by Hit Squad Project Controls &amp;C &amp;D &amp;R Page &amp;P of &amp;N</oddFooter>
@@ -2625,17 +3178,20 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr>
     <tabColor rgb="FF1F8A96"/>
-    <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:P8"/>
+  <dimension ref="A1:R14"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
-    <col min="1" max="1" width="32" customWidth="1"/>
-    <col min="2" max="6" width="12" customWidth="1"/>
-    <col min="7" max="16" width="14" customWidth="1"/>
+    <col min="1" max="1" width="28" customWidth="1"/>
+    <col min="2" max="2" width="14" customWidth="1"/>
+    <col min="3" max="3" width="26" customWidth="1"/>
+    <col min="4" max="5" width="14" customWidth="1"/>
+    <col min="6" max="10" width="12" customWidth="1"/>
+    <col min="11" max="11" width="14" customWidth="1"/>
+    <col min="12" max="18" width="7" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="22" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="1" ht="22" customHeight="1" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2654,13 +3210,15 @@
       <c r="N1" s="1"/>
       <c r="O1" s="1"/>
       <c r="P1" s="1"/>
+      <c r="Q1" s="1"/>
+      <c r="R1" s="1"/>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
         <v>2</v>
       </c>
@@ -2679,6 +3237,8 @@
       <c r="N3" s="3"/>
       <c r="O3" s="3"/>
       <c r="P3" s="3"/>
+      <c r="Q3" s="3"/>
+      <c r="R3" s="3"/>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A4" s="4" t="s">
@@ -2690,152 +3250,323 @@
         <v>4</v>
       </c>
       <c r="B5" s="6">
-        <v>46269.69564805555</v>
-      </c>
-    </row>
-    <row r="6" ht="20" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+        <v>46269.70988200232</v>
+      </c>
+    </row>
+    <row r="6" ht="20" customHeight="1" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A6" s="7" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="B6" s="7" t="s">
         <v>46</v>
       </c>
       <c r="C6" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="D6" s="7" t="s">
+        <v>47</v>
+      </c>
+      <c r="E6" s="7" t="s">
+        <v>48</v>
+      </c>
+      <c r="F6" s="7" t="s">
+        <v>49</v>
+      </c>
+      <c r="G6" s="7" t="s">
         <v>40</v>
       </c>
-      <c r="D6" s="7" t="s">
+      <c r="H6" s="7" t="s">
         <v>41</v>
       </c>
-      <c r="E6" s="7" t="s">
+      <c r="I6" s="7" t="s">
         <v>42</v>
       </c>
-      <c r="F6" s="7" t="s">
-        <v>47</v>
-      </c>
-      <c r="G6" s="7" t="s">
-        <v>48</v>
-      </c>
-      <c r="H6" s="7" t="s">
-        <v>49</v>
-      </c>
-      <c r="I6" s="7" t="s">
+      <c r="J6" s="7" t="s">
         <v>50</v>
       </c>
-      <c r="J6" s="7" t="s">
+      <c r="K6" s="7" t="s">
+        <v>12</v>
+      </c>
+      <c r="L6" s="22">
+        <v>46266</v>
+      </c>
+      <c r="M6" s="22">
+        <f>L6+1</f>
+      </c>
+      <c r="N6" s="22">
+        <f>M6+1</f>
+      </c>
+      <c r="O6" s="22">
+        <f>N6+1</f>
+      </c>
+      <c r="P6" s="22">
+        <f>O6+1</f>
+      </c>
+      <c r="Q6" s="22">
+        <f>P6+1</f>
+      </c>
+      <c r="R6" s="22">
+        <f>Q6+1</f>
+      </c>
+    </row>
+    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A7" s="23" t="s">
         <v>51</v>
       </c>
-      <c r="K6" s="7" t="s">
+      <c r="B7" s="24">
+        <f>G7+H7+I7</f>
+      </c>
+      <c r="C7" s="23" t="s">
+        <v>59</v>
+      </c>
+      <c r="D7" s="25">
+        <f>K7</f>
+      </c>
+      <c r="G7" s="24">
+        <f>B10</f>
+      </c>
+      <c r="H7" s="24">
+        <f>B11</f>
+      </c>
+      <c r="I7" s="24">
+        <f>B12</f>
+      </c>
+      <c r="J7" s="24">
+        <f>B13</f>
+      </c>
+      <c r="K7" s="25">
+        <f>D10+D11+D12</f>
+      </c>
+    </row>
+    <row r="8" spans="6:18" x14ac:dyDescent="0.25">
+      <c r="F8" s="26" t="s">
         <v>52</v>
       </c>
-      <c r="L6" s="7" t="s">
+      <c r="L8" s="27">
+        <v>1</v>
+      </c>
+      <c r="M8" s="27">
+        <v>1</v>
+      </c>
+      <c r="N8" s="27">
+        <v>1</v>
+      </c>
+      <c r="O8" s="27">
+        <v>1</v>
+      </c>
+      <c r="P8" s="27">
+        <v>1</v>
+      </c>
+      <c r="Q8" s="27">
+        <v>1</v>
+      </c>
+      <c r="R8" s="27">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A9" s="26" t="s">
         <v>53</v>
       </c>
-      <c r="M6" s="7" t="s">
+      <c r="F9" s="26" t="s">
         <v>54</v>
       </c>
-      <c r="N6" s="7" t="s">
+      <c r="L9" s="28">
+        <v>10</v>
+      </c>
+      <c r="M9" s="28">
+        <v>10</v>
+      </c>
+      <c r="N9" s="28">
+        <v>10</v>
+      </c>
+      <c r="O9" s="28">
+        <v>10</v>
+      </c>
+      <c r="P9" s="28">
+        <v>10</v>
+      </c>
+      <c r="Q9" s="28">
+        <v>10</v>
+      </c>
+      <c r="R9" s="28">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="10" spans="2:18" x14ac:dyDescent="0.25">
+      <c r="B10" s="21">
+        <f>SUM(L10:R10)</f>
+      </c>
+      <c r="D10" s="29">
+        <f>B10*E10</f>
+      </c>
+      <c r="E10" s="29">
+        <f>'Rate Tables'!C10</f>
+      </c>
+      <c r="F10" s="8" t="s">
         <v>55</v>
       </c>
-      <c r="O6" s="7" t="s">
+      <c r="L10" s="21">
+        <f>IF(L$6="","",IF(OR(WEEKDAY(L$6,1)=1,WEEKDAY(L$6,1)=7),0,MIN(8,L9)*L8))</f>
+      </c>
+      <c r="M10" s="21">
+        <f>IF(M$6="","",IF(OR(WEEKDAY(M$6,1)=1,WEEKDAY(M$6,1)=7),0,MIN(8,M9)*M8))</f>
+      </c>
+      <c r="N10" s="21">
+        <f>IF(N$6="","",IF(OR(WEEKDAY(N$6,1)=1,WEEKDAY(N$6,1)=7),0,MIN(8,N9)*N8))</f>
+      </c>
+      <c r="O10" s="21">
+        <f>IF(O$6="","",IF(OR(WEEKDAY(O$6,1)=1,WEEKDAY(O$6,1)=7),0,MIN(8,O9)*O8))</f>
+      </c>
+      <c r="P10" s="21">
+        <f>IF(P$6="","",IF(OR(WEEKDAY(P$6,1)=1,WEEKDAY(P$6,1)=7),0,MIN(8,P9)*P8))</f>
+      </c>
+      <c r="Q10" s="21">
+        <f>IF(Q$6="","",IF(OR(WEEKDAY(Q$6,1)=1,WEEKDAY(Q$6,1)=7),0,MIN(8,Q9)*Q8))</f>
+      </c>
+      <c r="R10" s="21">
+        <f>IF(R$6="","",IF(OR(WEEKDAY(R$6,1)=1,WEEKDAY(R$6,1)=7),0,MIN(8,R9)*R8))</f>
+      </c>
+    </row>
+    <row r="11" spans="2:18" x14ac:dyDescent="0.25">
+      <c r="B11" s="21">
+        <f>SUM(L11:R11)</f>
+      </c>
+      <c r="D11" s="29">
+        <f>B11*E11</f>
+      </c>
+      <c r="E11" s="29">
+        <f>'Rate Tables'!D10</f>
+      </c>
+      <c r="F11" s="8" t="s">
         <v>56</v>
       </c>
-      <c r="P6" s="7" t="s">
+      <c r="L11" s="21">
+        <f>IF(L$6="","",IF(WEEKDAY(L$6,1)=1,0,IF(WEEKDAY(L$6,1)=7,L9*L8,MAX(0,L9-8)*L8)))</f>
+      </c>
+      <c r="M11" s="21">
+        <f>IF(M$6="","",IF(WEEKDAY(M$6,1)=1,0,IF(WEEKDAY(M$6,1)=7,M9*M8,MAX(0,M9-8)*M8)))</f>
+      </c>
+      <c r="N11" s="21">
+        <f>IF(N$6="","",IF(WEEKDAY(N$6,1)=1,0,IF(WEEKDAY(N$6,1)=7,N9*N8,MAX(0,N9-8)*N8)))</f>
+      </c>
+      <c r="O11" s="21">
+        <f>IF(O$6="","",IF(WEEKDAY(O$6,1)=1,0,IF(WEEKDAY(O$6,1)=7,O9*O8,MAX(0,O9-8)*O8)))</f>
+      </c>
+      <c r="P11" s="21">
+        <f>IF(P$6="","",IF(WEEKDAY(P$6,1)=1,0,IF(WEEKDAY(P$6,1)=7,P9*P8,MAX(0,P9-8)*P8)))</f>
+      </c>
+      <c r="Q11" s="21">
+        <f>IF(Q$6="","",IF(WEEKDAY(Q$6,1)=1,0,IF(WEEKDAY(Q$6,1)=7,Q9*Q8,MAX(0,Q9-8)*Q8)))</f>
+      </c>
+      <c r="R11" s="21">
+        <f>IF(R$6="","",IF(WEEKDAY(R$6,1)=1,0,IF(WEEKDAY(R$6,1)=7,R9*R8,MAX(0,R9-8)*R8)))</f>
+      </c>
+    </row>
+    <row r="12" spans="2:18" x14ac:dyDescent="0.25">
+      <c r="B12" s="21">
+        <f>SUM(L12:R12)</f>
+      </c>
+      <c r="D12" s="29">
+        <f>B12*E12</f>
+      </c>
+      <c r="E12" s="29">
+        <f>'Rate Tables'!E10</f>
+      </c>
+      <c r="F12" s="8" t="s">
         <v>57</v>
       </c>
-    </row>
-    <row r="7" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A7" s="8" t="s">
+      <c r="L12" s="21">
+        <f>IF(L$6="","",IF(WEEKDAY(L$6,1)=1,L9*L8,0))</f>
+      </c>
+      <c r="M12" s="21">
+        <f>IF(M$6="","",IF(WEEKDAY(M$6,1)=1,M9*M8,0))</f>
+      </c>
+      <c r="N12" s="21">
+        <f>IF(N$6="","",IF(WEEKDAY(N$6,1)=1,N9*N8,0))</f>
+      </c>
+      <c r="O12" s="21">
+        <f>IF(O$6="","",IF(WEEKDAY(O$6,1)=1,O9*O8,0))</f>
+      </c>
+      <c r="P12" s="21">
+        <f>IF(P$6="","",IF(WEEKDAY(P$6,1)=1,P9*P8,0))</f>
+      </c>
+      <c r="Q12" s="21">
+        <f>IF(Q$6="","",IF(WEEKDAY(Q$6,1)=1,Q9*Q8,0))</f>
+      </c>
+      <c r="R12" s="21">
+        <f>IF(R$6="","",IF(WEEKDAY(R$6,1)=1,R9*R8,0))</f>
+      </c>
+    </row>
+    <row r="13" spans="2:18" x14ac:dyDescent="0.25">
+      <c r="B13" s="21">
+        <f>SUM(L13:R13)</f>
+      </c>
+      <c r="D13" s="29">
+        <f>B13*E13</f>
+      </c>
+      <c r="E13" s="29">
+        <v>130</v>
+      </c>
+      <c r="F13" s="8" t="s">
         <v>58</v>
       </c>
-      <c r="B7" s="19">
-        <v>1</v>
-      </c>
-      <c r="C7" s="21">
-        <v>8</v>
-      </c>
-      <c r="D7" s="21">
-        <v>2</v>
-      </c>
-      <c r="E7" s="21">
-        <v>0</v>
-      </c>
-      <c r="F7" s="21">
-        <v>1</v>
-      </c>
-      <c r="G7" s="22">
-        <f>'Rate Tables'!C10</f>
-      </c>
-      <c r="H7" s="22">
-        <f>'Rate Tables'!D10</f>
-      </c>
-      <c r="I7" s="22">
-        <f>'Rate Tables'!E10</f>
-      </c>
-      <c r="J7" s="22">
-        <v>130</v>
-      </c>
-      <c r="K7" s="22">
-        <f>C7*G7</f>
-      </c>
-      <c r="L7" s="22">
-        <f>D7*H7</f>
-      </c>
-      <c r="M7" s="22">
-        <f>E7*I7</f>
-      </c>
-      <c r="N7" s="22">
-        <f>F7*J7</f>
-      </c>
-      <c r="O7" s="22">
-        <f>K7+L7+M7</f>
-      </c>
-      <c r="P7" s="21">
-        <f>C7+D7+E7</f>
-      </c>
-    </row>
-    <row r="8" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A8" s="14" t="s">
+      <c r="L13" s="19">
+        <v>1</v>
+      </c>
+      <c r="M13" s="19">
+        <v>1</v>
+      </c>
+      <c r="N13" s="19">
+        <v>1</v>
+      </c>
+      <c r="O13" s="19">
+        <v>1</v>
+      </c>
+      <c r="P13" s="19">
+        <v>1</v>
+      </c>
+      <c r="Q13" s="19">
+        <v>1</v>
+      </c>
+      <c r="R13" s="19">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="14" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A14" s="14" t="s">
         <v>45</v>
       </c>
-      <c r="C8" s="15">
-        <f>SUM(C7:C7)</f>
-      </c>
-      <c r="D8" s="15">
-        <f>SUM(D7:D7)</f>
-      </c>
-      <c r="E8" s="15">
-        <f>SUM(E7:E7)</f>
-      </c>
-      <c r="F8" s="15">
-        <f>SUM(F7:F7)</f>
-      </c>
-      <c r="K8" s="18">
-        <f>SUM(K7:K7)</f>
-      </c>
-      <c r="L8" s="18">
-        <f>SUM(L7:L7)</f>
-      </c>
-      <c r="M8" s="18">
-        <f>SUM(M7:M7)</f>
-      </c>
-      <c r="N8" s="18">
-        <f>SUM(N7:N7)</f>
-      </c>
-      <c r="O8" s="18">
-        <f>SUM(O7:O7)</f>
-      </c>
-      <c r="P8" s="15">
-        <f>SUM(P7:P7)</f>
+      <c r="B14" s="15">
+        <f>SUM(B7)</f>
+      </c>
+      <c r="D14" s="18">
+        <f>SUM(D13)</f>
+      </c>
+      <c r="G14" s="15">
+        <f>SUM(G7)</f>
+      </c>
+      <c r="H14" s="15">
+        <f>SUM(H7)</f>
+      </c>
+      <c r="I14" s="15">
+        <f>SUM(I7)</f>
+      </c>
+      <c r="J14" s="15">
+        <f>SUM(J7)</f>
+      </c>
+      <c r="K14" s="18">
+        <f>SUM(K7)</f>
       </c>
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A1:P1"/>
-    <mergeCell ref="A3:P3"/>
+    <mergeCell ref="A1:R1"/>
+    <mergeCell ref="A3:R3"/>
   </mergeCells>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.4" right="0.4" top="0.65" bottom="0.65" header="0.28" footer="0.28"/>
-  <pageSetup orientation="landscape" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="20"/>
+  <pageSetup orientation="landscape" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100"/>
   <headerFooter>
     <oddHeader>&amp;L&amp;B HIT SQUAD / PROJECT CONTROLS &amp;C Direct &amp;R Confidential</oddHeader>
     <oddFooter>&amp;L Produced by Hit Squad Project Controls &amp;C &amp;D &amp;R Page &amp;P of &amp;N</oddFooter>
@@ -2849,17 +3580,20 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr>
     <tabColor rgb="FF1F8A96"/>
-    <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:P8"/>
+  <dimension ref="A1:R14"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
-    <col min="1" max="1" width="32" customWidth="1"/>
-    <col min="2" max="6" width="12" customWidth="1"/>
-    <col min="7" max="16" width="14" customWidth="1"/>
+    <col min="1" max="1" width="28" customWidth="1"/>
+    <col min="2" max="2" width="14" customWidth="1"/>
+    <col min="3" max="3" width="26" customWidth="1"/>
+    <col min="4" max="5" width="14" customWidth="1"/>
+    <col min="6" max="10" width="12" customWidth="1"/>
+    <col min="11" max="11" width="14" customWidth="1"/>
+    <col min="12" max="18" width="7" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="22" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="1" ht="22" customHeight="1" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2878,13 +3612,15 @@
       <c r="N1" s="1"/>
       <c r="O1" s="1"/>
       <c r="P1" s="1"/>
+      <c r="Q1" s="1"/>
+      <c r="R1" s="1"/>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
         <v>2</v>
       </c>
@@ -2903,6 +3639,8 @@
       <c r="N3" s="3"/>
       <c r="O3" s="3"/>
       <c r="P3" s="3"/>
+      <c r="Q3" s="3"/>
+      <c r="R3" s="3"/>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A4" s="4" t="s">
@@ -2914,152 +3652,323 @@
         <v>4</v>
       </c>
       <c r="B5" s="6">
-        <v>46269.69564805555</v>
-      </c>
-    </row>
-    <row r="6" ht="20" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+        <v>46269.70988201389</v>
+      </c>
+    </row>
+    <row r="6" ht="20" customHeight="1" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A6" s="7" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="B6" s="7" t="s">
         <v>46</v>
       </c>
       <c r="C6" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="D6" s="7" t="s">
+        <v>47</v>
+      </c>
+      <c r="E6" s="7" t="s">
+        <v>48</v>
+      </c>
+      <c r="F6" s="7" t="s">
+        <v>49</v>
+      </c>
+      <c r="G6" s="7" t="s">
         <v>40</v>
       </c>
-      <c r="D6" s="7" t="s">
+      <c r="H6" s="7" t="s">
         <v>41</v>
       </c>
-      <c r="E6" s="7" t="s">
+      <c r="I6" s="7" t="s">
         <v>42</v>
       </c>
-      <c r="F6" s="7" t="s">
-        <v>47</v>
-      </c>
-      <c r="G6" s="7" t="s">
-        <v>48</v>
-      </c>
-      <c r="H6" s="7" t="s">
-        <v>49</v>
-      </c>
-      <c r="I6" s="7" t="s">
+      <c r="J6" s="7" t="s">
         <v>50</v>
       </c>
-      <c r="J6" s="7" t="s">
+      <c r="K6" s="7" t="s">
+        <v>12</v>
+      </c>
+      <c r="L6" s="22">
+        <v>46266</v>
+      </c>
+      <c r="M6" s="22">
+        <f>L6+1</f>
+      </c>
+      <c r="N6" s="22">
+        <f>M6+1</f>
+      </c>
+      <c r="O6" s="22">
+        <f>N6+1</f>
+      </c>
+      <c r="P6" s="22">
+        <f>O6+1</f>
+      </c>
+      <c r="Q6" s="22">
+        <f>P6+1</f>
+      </c>
+      <c r="R6" s="22">
+        <f>Q6+1</f>
+      </c>
+    </row>
+    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A7" s="23" t="s">
         <v>51</v>
       </c>
-      <c r="K6" s="7" t="s">
+      <c r="B7" s="24">
+        <f>G7+H7+I7</f>
+      </c>
+      <c r="C7" s="23" t="s">
+        <v>60</v>
+      </c>
+      <c r="D7" s="25">
+        <f>K7</f>
+      </c>
+      <c r="G7" s="24">
+        <f>B10</f>
+      </c>
+      <c r="H7" s="24">
+        <f>B11</f>
+      </c>
+      <c r="I7" s="24">
+        <f>B12</f>
+      </c>
+      <c r="J7" s="24">
+        <f>B13</f>
+      </c>
+      <c r="K7" s="25">
+        <f>D10+D11+D12</f>
+      </c>
+    </row>
+    <row r="8" spans="6:18" x14ac:dyDescent="0.25">
+      <c r="F8" s="26" t="s">
         <v>52</v>
       </c>
-      <c r="L6" s="7" t="s">
+      <c r="L8" s="27">
+        <v>1</v>
+      </c>
+      <c r="M8" s="27">
+        <v>1</v>
+      </c>
+      <c r="N8" s="27">
+        <v>1</v>
+      </c>
+      <c r="O8" s="27">
+        <v>1</v>
+      </c>
+      <c r="P8" s="27">
+        <v>1</v>
+      </c>
+      <c r="Q8" s="27">
+        <v>1</v>
+      </c>
+      <c r="R8" s="27">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A9" s="26" t="s">
         <v>53</v>
       </c>
-      <c r="M6" s="7" t="s">
+      <c r="F9" s="26" t="s">
         <v>54</v>
       </c>
-      <c r="N6" s="7" t="s">
+      <c r="L9" s="28">
+        <v>10</v>
+      </c>
+      <c r="M9" s="28">
+        <v>10</v>
+      </c>
+      <c r="N9" s="28">
+        <v>10</v>
+      </c>
+      <c r="O9" s="28">
+        <v>10</v>
+      </c>
+      <c r="P9" s="28">
+        <v>10</v>
+      </c>
+      <c r="Q9" s="28">
+        <v>10</v>
+      </c>
+      <c r="R9" s="28">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="10" spans="2:18" x14ac:dyDescent="0.25">
+      <c r="B10" s="21">
+        <f>SUM(L10:R10)</f>
+      </c>
+      <c r="D10" s="29">
+        <f>B10*E10</f>
+      </c>
+      <c r="E10" s="29">
+        <f>'Rate Tables'!C10</f>
+      </c>
+      <c r="F10" s="8" t="s">
         <v>55</v>
       </c>
-      <c r="O6" s="7" t="s">
+      <c r="L10" s="21">
+        <f>IF(L$6="","",IF(OR(WEEKDAY(L$6,1)=1,WEEKDAY(L$6,1)=7),0,MIN(8,L9)*L8))</f>
+      </c>
+      <c r="M10" s="21">
+        <f>IF(M$6="","",IF(OR(WEEKDAY(M$6,1)=1,WEEKDAY(M$6,1)=7),0,MIN(8,M9)*M8))</f>
+      </c>
+      <c r="N10" s="21">
+        <f>IF(N$6="","",IF(OR(WEEKDAY(N$6,1)=1,WEEKDAY(N$6,1)=7),0,MIN(8,N9)*N8))</f>
+      </c>
+      <c r="O10" s="21">
+        <f>IF(O$6="","",IF(OR(WEEKDAY(O$6,1)=1,WEEKDAY(O$6,1)=7),0,MIN(8,O9)*O8))</f>
+      </c>
+      <c r="P10" s="21">
+        <f>IF(P$6="","",IF(OR(WEEKDAY(P$6,1)=1,WEEKDAY(P$6,1)=7),0,MIN(8,P9)*P8))</f>
+      </c>
+      <c r="Q10" s="21">
+        <f>IF(Q$6="","",IF(OR(WEEKDAY(Q$6,1)=1,WEEKDAY(Q$6,1)=7),0,MIN(8,Q9)*Q8))</f>
+      </c>
+      <c r="R10" s="21">
+        <f>IF(R$6="","",IF(OR(WEEKDAY(R$6,1)=1,WEEKDAY(R$6,1)=7),0,MIN(8,R9)*R8))</f>
+      </c>
+    </row>
+    <row r="11" spans="2:18" x14ac:dyDescent="0.25">
+      <c r="B11" s="21">
+        <f>SUM(L11:R11)</f>
+      </c>
+      <c r="D11" s="29">
+        <f>B11*E11</f>
+      </c>
+      <c r="E11" s="29">
+        <f>'Rate Tables'!D10</f>
+      </c>
+      <c r="F11" s="8" t="s">
         <v>56</v>
       </c>
-      <c r="P6" s="7" t="s">
+      <c r="L11" s="21">
+        <f>IF(L$6="","",IF(WEEKDAY(L$6,1)=1,0,IF(WEEKDAY(L$6,1)=7,L9*L8,MAX(0,L9-8)*L8)))</f>
+      </c>
+      <c r="M11" s="21">
+        <f>IF(M$6="","",IF(WEEKDAY(M$6,1)=1,0,IF(WEEKDAY(M$6,1)=7,M9*M8,MAX(0,M9-8)*M8)))</f>
+      </c>
+      <c r="N11" s="21">
+        <f>IF(N$6="","",IF(WEEKDAY(N$6,1)=1,0,IF(WEEKDAY(N$6,1)=7,N9*N8,MAX(0,N9-8)*N8)))</f>
+      </c>
+      <c r="O11" s="21">
+        <f>IF(O$6="","",IF(WEEKDAY(O$6,1)=1,0,IF(WEEKDAY(O$6,1)=7,O9*O8,MAX(0,O9-8)*O8)))</f>
+      </c>
+      <c r="P11" s="21">
+        <f>IF(P$6="","",IF(WEEKDAY(P$6,1)=1,0,IF(WEEKDAY(P$6,1)=7,P9*P8,MAX(0,P9-8)*P8)))</f>
+      </c>
+      <c r="Q11" s="21">
+        <f>IF(Q$6="","",IF(WEEKDAY(Q$6,1)=1,0,IF(WEEKDAY(Q$6,1)=7,Q9*Q8,MAX(0,Q9-8)*Q8)))</f>
+      </c>
+      <c r="R11" s="21">
+        <f>IF(R$6="","",IF(WEEKDAY(R$6,1)=1,0,IF(WEEKDAY(R$6,1)=7,R9*R8,MAX(0,R9-8)*R8)))</f>
+      </c>
+    </row>
+    <row r="12" spans="2:18" x14ac:dyDescent="0.25">
+      <c r="B12" s="21">
+        <f>SUM(L12:R12)</f>
+      </c>
+      <c r="D12" s="29">
+        <f>B12*E12</f>
+      </c>
+      <c r="E12" s="29">
+        <f>'Rate Tables'!E10</f>
+      </c>
+      <c r="F12" s="8" t="s">
         <v>57</v>
       </c>
-    </row>
-    <row r="7" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A7" s="8" t="s">
-        <v>59</v>
-      </c>
-      <c r="B7" s="19">
-        <v>1</v>
-      </c>
-      <c r="C7" s="21">
-        <v>8</v>
-      </c>
-      <c r="D7" s="21">
-        <v>2</v>
-      </c>
-      <c r="E7" s="21">
-        <v>0</v>
-      </c>
-      <c r="F7" s="21">
-        <v>1</v>
-      </c>
-      <c r="G7" s="22">
-        <f>'Rate Tables'!C10</f>
-      </c>
-      <c r="H7" s="22">
-        <f>'Rate Tables'!D10</f>
-      </c>
-      <c r="I7" s="22">
-        <f>'Rate Tables'!E10</f>
-      </c>
-      <c r="J7" s="22">
+      <c r="L12" s="21">
+        <f>IF(L$6="","",IF(WEEKDAY(L$6,1)=1,L9*L8,0))</f>
+      </c>
+      <c r="M12" s="21">
+        <f>IF(M$6="","",IF(WEEKDAY(M$6,1)=1,M9*M8,0))</f>
+      </c>
+      <c r="N12" s="21">
+        <f>IF(N$6="","",IF(WEEKDAY(N$6,1)=1,N9*N8,0))</f>
+      </c>
+      <c r="O12" s="21">
+        <f>IF(O$6="","",IF(WEEKDAY(O$6,1)=1,O9*O8,0))</f>
+      </c>
+      <c r="P12" s="21">
+        <f>IF(P$6="","",IF(WEEKDAY(P$6,1)=1,P9*P8,0))</f>
+      </c>
+      <c r="Q12" s="21">
+        <f>IF(Q$6="","",IF(WEEKDAY(Q$6,1)=1,Q9*Q8,0))</f>
+      </c>
+      <c r="R12" s="21">
+        <f>IF(R$6="","",IF(WEEKDAY(R$6,1)=1,R9*R8,0))</f>
+      </c>
+    </row>
+    <row r="13" spans="2:18" x14ac:dyDescent="0.25">
+      <c r="B13" s="21">
+        <f>SUM(L13:R13)</f>
+      </c>
+      <c r="D13" s="29">
+        <f>B13*E13</f>
+      </c>
+      <c r="E13" s="29">
         <v>130</v>
       </c>
-      <c r="K7" s="22">
-        <f>C7*G7</f>
-      </c>
-      <c r="L7" s="22">
-        <f>D7*H7</f>
-      </c>
-      <c r="M7" s="22">
-        <f>E7*I7</f>
-      </c>
-      <c r="N7" s="22">
-        <f>F7*J7</f>
-      </c>
-      <c r="O7" s="22">
-        <f>K7+L7+M7</f>
-      </c>
-      <c r="P7" s="21">
-        <f>C7+D7+E7</f>
-      </c>
-    </row>
-    <row r="8" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A8" s="14" t="s">
+      <c r="F13" s="8" t="s">
+        <v>58</v>
+      </c>
+      <c r="L13" s="19">
+        <v>1</v>
+      </c>
+      <c r="M13" s="19">
+        <v>1</v>
+      </c>
+      <c r="N13" s="19">
+        <v>1</v>
+      </c>
+      <c r="O13" s="19">
+        <v>1</v>
+      </c>
+      <c r="P13" s="19">
+        <v>1</v>
+      </c>
+      <c r="Q13" s="19">
+        <v>1</v>
+      </c>
+      <c r="R13" s="19">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="14" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A14" s="14" t="s">
         <v>45</v>
       </c>
-      <c r="C8" s="15">
-        <f>SUM(C7:C7)</f>
-      </c>
-      <c r="D8" s="15">
-        <f>SUM(D7:D7)</f>
-      </c>
-      <c r="E8" s="15">
-        <f>SUM(E7:E7)</f>
-      </c>
-      <c r="F8" s="15">
-        <f>SUM(F7:F7)</f>
-      </c>
-      <c r="K8" s="18">
-        <f>SUM(K7:K7)</f>
-      </c>
-      <c r="L8" s="18">
-        <f>SUM(L7:L7)</f>
-      </c>
-      <c r="M8" s="18">
-        <f>SUM(M7:M7)</f>
-      </c>
-      <c r="N8" s="18">
-        <f>SUM(N7:N7)</f>
-      </c>
-      <c r="O8" s="18">
-        <f>SUM(O7:O7)</f>
-      </c>
-      <c r="P8" s="15">
-        <f>SUM(P7:P7)</f>
+      <c r="B14" s="15">
+        <f>SUM(B7)</f>
+      </c>
+      <c r="D14" s="18">
+        <f>SUM(D13)</f>
+      </c>
+      <c r="G14" s="15">
+        <f>SUM(G7)</f>
+      </c>
+      <c r="H14" s="15">
+        <f>SUM(H7)</f>
+      </c>
+      <c r="I14" s="15">
+        <f>SUM(I7)</f>
+      </c>
+      <c r="J14" s="15">
+        <f>SUM(J7)</f>
+      </c>
+      <c r="K14" s="18">
+        <f>SUM(K7)</f>
       </c>
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A1:P1"/>
-    <mergeCell ref="A3:P3"/>
+    <mergeCell ref="A1:R1"/>
+    <mergeCell ref="A3:R3"/>
   </mergeCells>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.4" right="0.4" top="0.65" bottom="0.65" header="0.28" footer="0.28"/>
-  <pageSetup orientation="landscape" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="20"/>
+  <pageSetup orientation="landscape" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100"/>
   <headerFooter>
     <oddHeader>&amp;L&amp;B HIT SQUAD / PROJECT CONTROLS &amp;C Support &amp;R Confidential</oddHeader>
     <oddFooter>&amp;L Produced by Hit Squad Project Controls &amp;C &amp;D &amp;R Page &amp;P of &amp;N</oddFooter>
@@ -3122,58 +4031,58 @@
         <v>4</v>
       </c>
       <c r="B5" s="6">
-        <v>46269.69564805555</v>
+        <v>46269.70988201389</v>
       </c>
     </row>
     <row r="6" ht="20" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A6" s="7" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="B6" s="7" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="C6" s="7" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="D6" s="7" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="E6" s="7" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="F6" s="7" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="G6" s="7" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="H6" s="7" t="s">
-        <v>56</v>
+        <v>68</v>
       </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A7" s="8" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="B7" s="8" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="C7" s="19">
         <v>1</v>
       </c>
       <c r="D7" s="19">
-        <v>1</v>
-      </c>
-      <c r="E7" s="22">
+        <v>7</v>
+      </c>
+      <c r="E7" s="29">
         <v>134</v>
       </c>
-      <c r="F7" s="22">
+      <c r="F7" s="29">
         <v>0</v>
       </c>
-      <c r="G7" s="22">
+      <c r="G7" s="29">
         <f>C7*D7*E7+F7</f>
       </c>
-      <c r="H7" s="22">
+      <c r="H7" s="29">
         <f>G7*1.06</f>
       </c>
     </row>
@@ -3258,58 +4167,58 @@
         <v>4</v>
       </c>
       <c r="B5" s="6">
-        <v>46269.69564805555</v>
+        <v>46269.70988201389</v>
       </c>
     </row>
     <row r="6" ht="20" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A6" s="7" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="B6" s="7" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="C6" s="7" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="D6" s="7" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="E6" s="7" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="F6" s="7" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="G6" s="7" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="H6" s="7" t="s">
-        <v>56</v>
+        <v>68</v>
       </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A7" s="8" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="B7" s="8" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="C7" s="19">
         <v>1</v>
       </c>
       <c r="D7" s="19">
-        <v>1</v>
-      </c>
-      <c r="E7" s="22">
+        <v>7</v>
+      </c>
+      <c r="E7" s="29">
         <v>80</v>
       </c>
-      <c r="F7" s="22">
+      <c r="F7" s="29">
         <v>0</v>
       </c>
-      <c r="G7" s="22">
+      <c r="G7" s="29">
         <f>C7*D7*E7+F7</f>
       </c>
-      <c r="H7" s="22">
+      <c r="H7" s="29">
         <f>G7*1.06</f>
       </c>
     </row>

</xml_diff>

<commit_message>
Lock daily labor grid as a stable edit surface
Keep Staff/Foremen/Direct/Support as 7-row workbook blocks with Type labels TITLE/HC/HPS/ST/OT/DT/PD and a hidden block-id column for a later importer. No import UI. Regenerated Look samples.

Co-authored-by: robertmhenderson582-ops <robertmhenderson582-ops@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/look-samples/v151_2027_aromatics_client_package.xlsx
+++ b/look-samples/v151_2027_aromatics_client_package.xlsx
@@ -60,7 +60,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="295" uniqueCount="96">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="335" uniqueCount="102">
   <si>
     <t>HIT SQUAD / PROJECT CONTROLS</t>
   </si>
@@ -218,6 +218,12 @@
     <t>DAYSHIFT</t>
   </si>
   <si>
+    <t>TITLE</t>
+  </si>
+  <si>
+    <t>st-1|day</t>
+  </si>
+  <si>
     <t>HC</t>
   </si>
   <si>
@@ -239,10 +245,22 @@
     <t>PD</t>
   </si>
   <si>
+    <t>gf-1|day</t>
+  </si>
+  <si>
+    <t>fm-1|day</t>
+  </si>
+  <si>
     <t>Boilermaker Journeyman</t>
   </si>
   <si>
+    <t>dr-1|day</t>
+  </si>
+  <si>
     <t>Fire Watch</t>
+  </si>
+  <si>
+    <t>su-1|day</t>
   </si>
   <si>
     <t>Item</t>
@@ -913,7 +931,7 @@
         <v>4</v>
       </c>
       <c r="B5" s="6">
-        <v>46269.70988202546</v>
+        <v>46269.71300210648</v>
       </c>
     </row>
     <row r="6" ht="20" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
@@ -1144,41 +1162,41 @@
         <v>4</v>
       </c>
       <c r="B5" s="6">
-        <v>46269.70988201389</v>
+        <v>46269.71300208333</v>
       </c>
     </row>
     <row r="6" ht="20" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A6" s="7" t="s">
-        <v>61</v>
+        <v>67</v>
       </c>
       <c r="B6" s="7" t="s">
-        <v>62</v>
+        <v>68</v>
       </c>
       <c r="C6" s="7" t="s">
-        <v>63</v>
+        <v>69</v>
       </c>
       <c r="D6" s="7" t="s">
-        <v>64</v>
+        <v>70</v>
       </c>
       <c r="E6" s="7" t="s">
-        <v>65</v>
+        <v>71</v>
       </c>
       <c r="F6" s="7" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="G6" s="7" t="s">
-        <v>67</v>
+        <v>73</v>
       </c>
       <c r="H6" s="7" t="s">
-        <v>68</v>
+        <v>74</v>
       </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A7" s="8" t="s">
-        <v>72</v>
+        <v>78</v>
       </c>
       <c r="B7" s="8" t="s">
-        <v>70</v>
+        <v>76</v>
       </c>
       <c r="C7" s="19">
         <v>1</v>
@@ -1283,41 +1301,41 @@
         <v>4</v>
       </c>
       <c r="B5" s="6">
-        <v>46269.70988202546</v>
+        <v>46269.71300210648</v>
       </c>
     </row>
     <row r="6" ht="20" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A6" s="7" t="s">
+        <v>79</v>
+      </c>
+      <c r="B6" s="7" t="s">
+        <v>80</v>
+      </c>
+      <c r="C6" s="7" t="s">
+        <v>69</v>
+      </c>
+      <c r="D6" s="7" t="s">
+        <v>71</v>
+      </c>
+      <c r="E6" s="7" t="s">
+        <v>81</v>
+      </c>
+      <c r="F6" s="7" t="s">
         <v>73</v>
       </c>
-      <c r="B6" s="7" t="s">
+      <c r="G6" s="7" t="s">
+        <v>82</v>
+      </c>
+      <c r="H6" s="7" t="s">
         <v>74</v>
-      </c>
-      <c r="C6" s="7" t="s">
-        <v>63</v>
-      </c>
-      <c r="D6" s="7" t="s">
-        <v>65</v>
-      </c>
-      <c r="E6" s="7" t="s">
-        <v>75</v>
-      </c>
-      <c r="F6" s="7" t="s">
-        <v>67</v>
-      </c>
-      <c r="G6" s="7" t="s">
-        <v>76</v>
-      </c>
-      <c r="H6" s="7" t="s">
-        <v>68</v>
       </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A7" s="8" t="s">
-        <v>77</v>
+        <v>83</v>
       </c>
       <c r="B7" s="8" t="s">
-        <v>78</v>
+        <v>84</v>
       </c>
       <c r="C7" s="19">
         <v>1</v>
@@ -1326,7 +1344,7 @@
         <v>500</v>
       </c>
       <c r="E7" s="8" t="s">
-        <v>79</v>
+        <v>85</v>
       </c>
       <c r="F7" s="29">
         <f>C7*D7</f>
@@ -1420,38 +1438,38 @@
         <v>4</v>
       </c>
       <c r="B5" s="6">
-        <v>46269.70988202546</v>
+        <v>46269.71300209491</v>
       </c>
     </row>
     <row r="6" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" s="7" t="s">
-        <v>61</v>
+        <v>67</v>
       </c>
       <c r="B6" s="7" t="s">
-        <v>62</v>
+        <v>68</v>
       </c>
       <c r="C6" s="7" t="s">
-        <v>63</v>
+        <v>69</v>
       </c>
       <c r="D6" s="7" t="s">
-        <v>64</v>
+        <v>70</v>
       </c>
       <c r="E6" s="7" t="s">
-        <v>65</v>
+        <v>71</v>
       </c>
       <c r="F6" s="7" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="G6" s="7" t="s">
-        <v>68</v>
+        <v>74</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" s="8" t="s">
-        <v>80</v>
+        <v>86</v>
       </c>
       <c r="B7" s="8" t="s">
-        <v>70</v>
+        <v>76</v>
       </c>
       <c r="C7" s="19">
         <v>1</v>
@@ -1541,29 +1559,29 @@
         <v>4</v>
       </c>
       <c r="B5" s="6">
-        <v>46269.70988202546</v>
+        <v>46269.71300210648</v>
       </c>
     </row>
     <row r="6" ht="20" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" s="7" t="s">
-        <v>81</v>
+        <v>87</v>
       </c>
       <c r="B6" s="7" t="s">
-        <v>82</v>
+        <v>88</v>
       </c>
       <c r="C6" s="7" t="s">
-        <v>83</v>
+        <v>89</v>
       </c>
       <c r="D6" s="7" t="s">
-        <v>84</v>
+        <v>90</v>
       </c>
       <c r="E6" s="7" t="s">
-        <v>68</v>
+        <v>74</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" s="8" t="s">
-        <v>85</v>
+        <v>91</v>
       </c>
       <c r="B7" s="19">
         <v>1</v>
@@ -1651,32 +1669,32 @@
         <v>4</v>
       </c>
       <c r="B5" s="6">
-        <v>46269.70988202546</v>
+        <v>46269.71300210648</v>
       </c>
     </row>
     <row r="6" ht="20" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" s="7" t="s">
-        <v>61</v>
+        <v>67</v>
       </c>
       <c r="B6" s="7" t="s">
-        <v>86</v>
+        <v>92</v>
       </c>
       <c r="C6" s="7" t="s">
-        <v>63</v>
+        <v>69</v>
       </c>
       <c r="D6" s="7" t="s">
-        <v>87</v>
+        <v>93</v>
       </c>
       <c r="E6" s="7" t="s">
-        <v>68</v>
+        <v>74</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" s="8" t="s">
-        <v>88</v>
+        <v>94</v>
       </c>
       <c r="B7" s="8" t="s">
-        <v>89</v>
+        <v>95</v>
       </c>
       <c r="C7" s="19">
         <v>1</v>
@@ -1761,27 +1779,27 @@
         <v>4</v>
       </c>
       <c r="B5" s="6">
-        <v>46269.70988199074</v>
+        <v>46269.71300206018</v>
       </c>
     </row>
     <row r="6" ht="20" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" s="7" t="s">
-        <v>90</v>
+        <v>96</v>
       </c>
       <c r="B6" s="7" t="s">
-        <v>91</v>
+        <v>97</v>
       </c>
       <c r="C6" s="7" t="s">
-        <v>92</v>
+        <v>98</v>
       </c>
       <c r="D6" s="7" t="s">
-        <v>93</v>
+        <v>99</v>
       </c>
       <c r="E6" s="7" t="s">
-        <v>94</v>
+        <v>100</v>
       </c>
       <c r="F6" s="7" t="s">
-        <v>95</v>
+        <v>101</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.25">
@@ -1846,7 +1864,7 @@
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10" s="8" t="s">
-        <v>59</v>
+        <v>63</v>
       </c>
       <c r="B10" s="29">
         <v>45.6</v>
@@ -1929,7 +1947,7 @@
         <v>4</v>
       </c>
       <c r="B5" s="6">
-        <v>46269.70988201389</v>
+        <v>46269.71300207176</v>
       </c>
     </row>
     <row r="6" ht="20" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -2075,7 +2093,7 @@
         <v>4</v>
       </c>
       <c r="B5" s="6">
-        <v>46269.70988201389</v>
+        <v>46269.71300207176</v>
       </c>
     </row>
     <row r="6" ht="20" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -2151,7 +2169,7 @@
   <sheetPr>
     <tabColor rgb="FF1F8A96"/>
   </sheetPr>
-  <dimension ref="A1:R21"/>
+  <dimension ref="A1:CX21"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="28" customWidth="1"/>
@@ -2161,6 +2179,7 @@
     <col min="6" max="10" width="12" customWidth="1"/>
     <col min="11" max="11" width="14" customWidth="1"/>
     <col min="12" max="18" width="7" customWidth="1"/>
+    <col min="102" max="102" width="3" hidden="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="22" customHeight="1" spans="1:18" x14ac:dyDescent="0.25">
@@ -2222,7 +2241,7 @@
         <v>4</v>
       </c>
       <c r="B5" s="6">
-        <v>46269.70988200232</v>
+        <v>46269.71300206018</v>
       </c>
     </row>
     <row r="6" ht="20" customHeight="1" spans="1:18" x14ac:dyDescent="0.25">
@@ -2281,7 +2300,7 @@
         <f>Q6+1</f>
       </c>
     </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:102" x14ac:dyDescent="0.25">
       <c r="A7" s="23" t="s">
         <v>51</v>
       </c>
@@ -2294,6 +2313,9 @@
       <c r="D7" s="25">
         <f>K7</f>
       </c>
+      <c r="F7" s="23" t="s">
+        <v>52</v>
+      </c>
       <c r="G7" s="24">
         <f>B10</f>
       </c>
@@ -2309,10 +2331,13 @@
       <c r="K7" s="25">
         <f>D10+D11+D12</f>
       </c>
-    </row>
-    <row r="8" spans="6:18" x14ac:dyDescent="0.25">
+      <c r="CX7" s="23" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="8" spans="6:102" x14ac:dyDescent="0.25">
       <c r="F8" s="26" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="L8" s="27">
         <v>1</v>
@@ -2335,13 +2360,16 @@
       <c r="R8" s="27">
         <v>1</v>
       </c>
-    </row>
-    <row r="9" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="CX8" s="26" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="9" spans="1:102" x14ac:dyDescent="0.25">
       <c r="A9" s="26" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="F9" s="26" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="L9" s="28">
         <v>10</v>
@@ -2364,8 +2392,11 @@
       <c r="R9" s="28">
         <v>10</v>
       </c>
-    </row>
-    <row r="10" spans="2:18" x14ac:dyDescent="0.25">
+      <c r="CX9" s="26" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="10" spans="2:102" x14ac:dyDescent="0.25">
       <c r="B10" s="21">
         <f>SUM(L10:R10)</f>
       </c>
@@ -2376,7 +2407,7 @@
         <f>'Rate Tables'!C7</f>
       </c>
       <c r="F10" s="8" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="L10" s="21">
         <f>IF(L$6="","",IF(WEEKDAY(L$6,1)=1,0,MIN(10,L9)*L8))</f>
@@ -2399,8 +2430,11 @@
       <c r="R10" s="21">
         <f>IF(R$6="","",IF(WEEKDAY(R$6,1)=1,0,MIN(10,R9)*R8))</f>
       </c>
-    </row>
-    <row r="11" spans="2:18" x14ac:dyDescent="0.25">
+      <c r="CX10" s="8" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="11" spans="2:102" x14ac:dyDescent="0.25">
       <c r="B11" s="21">
         <f>SUM(L11:R11)</f>
       </c>
@@ -2411,7 +2445,7 @@
         <f>'Rate Tables'!D7</f>
       </c>
       <c r="F11" s="8" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="L11" s="21">
         <f>IF(L$6="","",IF(WEEKDAY(L$6,1)=1,0,MAX(0,L9-10)*L8))</f>
@@ -2434,8 +2468,11 @@
       <c r="R11" s="21">
         <f>IF(R$6="","",IF(WEEKDAY(R$6,1)=1,0,MAX(0,R9-10)*R8))</f>
       </c>
-    </row>
-    <row r="12" spans="2:18" x14ac:dyDescent="0.25">
+      <c r="CX11" s="8" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="12" spans="2:102" x14ac:dyDescent="0.25">
       <c r="B12" s="21">
         <f>SUM(L12:R12)</f>
       </c>
@@ -2446,7 +2483,7 @@
         <f>'Rate Tables'!E7</f>
       </c>
       <c r="F12" s="8" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="L12" s="21">
         <f>IF(L$6="","",IF(WEEKDAY(L$6,1)=1,L9*L8,0))</f>
@@ -2469,8 +2506,11 @@
       <c r="R12" s="21">
         <f>IF(R$6="","",IF(WEEKDAY(R$6,1)=1,R9*R8,0))</f>
       </c>
-    </row>
-    <row r="13" spans="2:18" x14ac:dyDescent="0.25">
+      <c r="CX12" s="8" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="13" spans="2:102" x14ac:dyDescent="0.25">
       <c r="B13" s="21">
         <f>SUM(L13:R13)</f>
       </c>
@@ -2481,7 +2521,7 @@
         <v>140</v>
       </c>
       <c r="F13" s="8" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="L13" s="19">
         <v>1</v>
@@ -2504,8 +2544,11 @@
       <c r="R13" s="19">
         <v>1</v>
       </c>
-    </row>
-    <row r="14" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="CX13" s="8" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="14" spans="1:102" x14ac:dyDescent="0.25">
       <c r="A14" s="23" t="s">
         <v>51</v>
       </c>
@@ -2518,6 +2561,9 @@
       <c r="D14" s="25">
         <f>K14</f>
       </c>
+      <c r="F14" s="23" t="s">
+        <v>52</v>
+      </c>
       <c r="G14" s="24">
         <f>B17</f>
       </c>
@@ -2533,10 +2579,13 @@
       <c r="K14" s="25">
         <f>D17+D18+D19</f>
       </c>
-    </row>
-    <row r="15" spans="6:18" x14ac:dyDescent="0.25">
+      <c r="CX14" s="23" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="15" spans="6:102" x14ac:dyDescent="0.25">
       <c r="F15" s="26" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="L15" s="27">
         <v>1</v>
@@ -2559,13 +2608,16 @@
       <c r="R15" s="27">
         <v>1</v>
       </c>
-    </row>
-    <row r="16" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="CX15" s="26" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="16" spans="1:102" x14ac:dyDescent="0.25">
       <c r="A16" s="26" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="F16" s="26" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="L16" s="28">
         <v>10</v>
@@ -2588,8 +2640,11 @@
       <c r="R16" s="28">
         <v>10</v>
       </c>
-    </row>
-    <row r="17" spans="2:18" x14ac:dyDescent="0.25">
+      <c r="CX16" s="26" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="17" spans="2:102" x14ac:dyDescent="0.25">
       <c r="B17" s="21">
         <f>SUM(L17:R17)</f>
       </c>
@@ -2600,7 +2655,7 @@
         <f>'Rate Tables'!C8</f>
       </c>
       <c r="F17" s="8" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="L17" s="21">
         <f>IF(L$6="","",IF(OR(WEEKDAY(L$6,1)=1,WEEKDAY(L$6,1)=7),0,MIN(8,L16)*L15))</f>
@@ -2623,8 +2678,11 @@
       <c r="R17" s="21">
         <f>IF(R$6="","",IF(OR(WEEKDAY(R$6,1)=1,WEEKDAY(R$6,1)=7),0,MIN(8,R16)*R15))</f>
       </c>
-    </row>
-    <row r="18" spans="2:18" x14ac:dyDescent="0.25">
+      <c r="CX17" s="8" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="18" spans="2:102" x14ac:dyDescent="0.25">
       <c r="B18" s="21">
         <f>SUM(L18:R18)</f>
       </c>
@@ -2635,7 +2693,7 @@
         <f>'Rate Tables'!D8</f>
       </c>
       <c r="F18" s="8" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="L18" s="21">
         <f>IF(L$6="","",IF(WEEKDAY(L$6,1)=1,0,IF(WEEKDAY(L$6,1)=7,L16*L15,MAX(0,L16-8)*L15)))</f>
@@ -2658,8 +2716,11 @@
       <c r="R18" s="21">
         <f>IF(R$6="","",IF(WEEKDAY(R$6,1)=1,0,IF(WEEKDAY(R$6,1)=7,R16*R15,MAX(0,R16-8)*R15)))</f>
       </c>
-    </row>
-    <row r="19" spans="2:18" x14ac:dyDescent="0.25">
+      <c r="CX18" s="8" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="19" spans="2:102" x14ac:dyDescent="0.25">
       <c r="B19" s="21">
         <f>SUM(L19:R19)</f>
       </c>
@@ -2670,7 +2731,7 @@
         <f>'Rate Tables'!E8</f>
       </c>
       <c r="F19" s="8" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="L19" s="21">
         <f>IF(L$6="","",IF(WEEKDAY(L$6,1)=1,L16*L15,0))</f>
@@ -2693,8 +2754,11 @@
       <c r="R19" s="21">
         <f>IF(R$6="","",IF(WEEKDAY(R$6,1)=1,R16*R15,0))</f>
       </c>
-    </row>
-    <row r="20" spans="2:18" x14ac:dyDescent="0.25">
+      <c r="CX19" s="8" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="20" spans="2:102" x14ac:dyDescent="0.25">
       <c r="B20" s="21">
         <f>SUM(L20:R20)</f>
       </c>
@@ -2705,7 +2769,7 @@
         <v>140</v>
       </c>
       <c r="F20" s="8" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="L20" s="19">
         <v>1</v>
@@ -2727,6 +2791,9 @@
       </c>
       <c r="R20" s="19">
         <v>1</v>
+      </c>
+      <c r="CX20" s="8" t="s">
+        <v>61</v>
       </c>
     </row>
     <row r="21" spans="1:11" x14ac:dyDescent="0.25">
@@ -2777,7 +2844,7 @@
   <sheetPr>
     <tabColor rgb="FF1F8A96"/>
   </sheetPr>
-  <dimension ref="A1:R14"/>
+  <dimension ref="A1:CX14"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="28" customWidth="1"/>
@@ -2787,6 +2854,7 @@
     <col min="6" max="10" width="12" customWidth="1"/>
     <col min="11" max="11" width="14" customWidth="1"/>
     <col min="12" max="18" width="7" customWidth="1"/>
+    <col min="102" max="102" width="3" hidden="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="22" customHeight="1" spans="1:18" x14ac:dyDescent="0.25">
@@ -2848,7 +2916,7 @@
         <v>4</v>
       </c>
       <c r="B5" s="6">
-        <v>46269.70988200232</v>
+        <v>46269.71300207176</v>
       </c>
     </row>
     <row r="6" ht="20" customHeight="1" spans="1:18" x14ac:dyDescent="0.25">
@@ -2907,7 +2975,7 @@
         <f>Q6+1</f>
       </c>
     </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:102" x14ac:dyDescent="0.25">
       <c r="A7" s="23" t="s">
         <v>51</v>
       </c>
@@ -2920,6 +2988,9 @@
       <c r="D7" s="25">
         <f>K7</f>
       </c>
+      <c r="F7" s="23" t="s">
+        <v>52</v>
+      </c>
       <c r="G7" s="24">
         <f>B10</f>
       </c>
@@ -2935,10 +3006,13 @@
       <c r="K7" s="25">
         <f>D10+D11+D12</f>
       </c>
-    </row>
-    <row r="8" spans="6:18" x14ac:dyDescent="0.25">
+      <c r="CX7" s="23" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="8" spans="6:102" x14ac:dyDescent="0.25">
       <c r="F8" s="26" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="L8" s="27">
         <v>1</v>
@@ -2961,13 +3035,16 @@
       <c r="R8" s="27">
         <v>1</v>
       </c>
-    </row>
-    <row r="9" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="CX8" s="26" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="9" spans="1:102" x14ac:dyDescent="0.25">
       <c r="A9" s="26" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="F9" s="26" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="L9" s="28">
         <v>10</v>
@@ -2990,8 +3067,11 @@
       <c r="R9" s="28">
         <v>10</v>
       </c>
-    </row>
-    <row r="10" spans="2:18" x14ac:dyDescent="0.25">
+      <c r="CX9" s="26" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="10" spans="2:102" x14ac:dyDescent="0.25">
       <c r="B10" s="21">
         <f>SUM(L10:R10)</f>
       </c>
@@ -3002,7 +3082,7 @@
         <f>'Rate Tables'!C9</f>
       </c>
       <c r="F10" s="8" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="L10" s="21">
         <f>IF(L$6="","",IF(OR(WEEKDAY(L$6,1)=1,WEEKDAY(L$6,1)=7),0,MIN(8,L9)*L8))</f>
@@ -3025,8 +3105,11 @@
       <c r="R10" s="21">
         <f>IF(R$6="","",IF(OR(WEEKDAY(R$6,1)=1,WEEKDAY(R$6,1)=7),0,MIN(8,R9)*R8))</f>
       </c>
-    </row>
-    <row r="11" spans="2:18" x14ac:dyDescent="0.25">
+      <c r="CX10" s="8" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="11" spans="2:102" x14ac:dyDescent="0.25">
       <c r="B11" s="21">
         <f>SUM(L11:R11)</f>
       </c>
@@ -3037,7 +3120,7 @@
         <f>'Rate Tables'!D9</f>
       </c>
       <c r="F11" s="8" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="L11" s="21">
         <f>IF(L$6="","",IF(WEEKDAY(L$6,1)=1,0,IF(WEEKDAY(L$6,1)=7,L9*L8,MAX(0,L9-8)*L8)))</f>
@@ -3060,8 +3143,11 @@
       <c r="R11" s="21">
         <f>IF(R$6="","",IF(WEEKDAY(R$6,1)=1,0,IF(WEEKDAY(R$6,1)=7,R9*R8,MAX(0,R9-8)*R8)))</f>
       </c>
-    </row>
-    <row r="12" spans="2:18" x14ac:dyDescent="0.25">
+      <c r="CX11" s="8" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="12" spans="2:102" x14ac:dyDescent="0.25">
       <c r="B12" s="21">
         <f>SUM(L12:R12)</f>
       </c>
@@ -3072,7 +3158,7 @@
         <f>'Rate Tables'!E9</f>
       </c>
       <c r="F12" s="8" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="L12" s="21">
         <f>IF(L$6="","",IF(WEEKDAY(L$6,1)=1,L9*L8,0))</f>
@@ -3095,8 +3181,11 @@
       <c r="R12" s="21">
         <f>IF(R$6="","",IF(WEEKDAY(R$6,1)=1,R9*R8,0))</f>
       </c>
-    </row>
-    <row r="13" spans="2:18" x14ac:dyDescent="0.25">
+      <c r="CX12" s="8" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="13" spans="2:102" x14ac:dyDescent="0.25">
       <c r="B13" s="21">
         <f>SUM(L13:R13)</f>
       </c>
@@ -3107,7 +3196,7 @@
         <v>130</v>
       </c>
       <c r="F13" s="8" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="L13" s="19">
         <v>1</v>
@@ -3129,6 +3218,9 @@
       </c>
       <c r="R13" s="19">
         <v>1</v>
+      </c>
+      <c r="CX13" s="8" t="s">
+        <v>62</v>
       </c>
     </row>
     <row r="14" spans="1:11" x14ac:dyDescent="0.25">
@@ -3179,7 +3271,7 @@
   <sheetPr>
     <tabColor rgb="FF1F8A96"/>
   </sheetPr>
-  <dimension ref="A1:R14"/>
+  <dimension ref="A1:CX14"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="28" customWidth="1"/>
@@ -3189,6 +3281,7 @@
     <col min="6" max="10" width="12" customWidth="1"/>
     <col min="11" max="11" width="14" customWidth="1"/>
     <col min="12" max="18" width="7" customWidth="1"/>
+    <col min="102" max="102" width="3" hidden="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="22" customHeight="1" spans="1:18" x14ac:dyDescent="0.25">
@@ -3250,7 +3343,7 @@
         <v>4</v>
       </c>
       <c r="B5" s="6">
-        <v>46269.70988200232</v>
+        <v>46269.71300207176</v>
       </c>
     </row>
     <row r="6" ht="20" customHeight="1" spans="1:18" x14ac:dyDescent="0.25">
@@ -3309,7 +3402,7 @@
         <f>Q6+1</f>
       </c>
     </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:102" x14ac:dyDescent="0.25">
       <c r="A7" s="23" t="s">
         <v>51</v>
       </c>
@@ -3317,11 +3410,14 @@
         <f>G7+H7+I7</f>
       </c>
       <c r="C7" s="23" t="s">
-        <v>59</v>
+        <v>63</v>
       </c>
       <c r="D7" s="25">
         <f>K7</f>
       </c>
+      <c r="F7" s="23" t="s">
+        <v>52</v>
+      </c>
       <c r="G7" s="24">
         <f>B10</f>
       </c>
@@ -3337,10 +3433,13 @@
       <c r="K7" s="25">
         <f>D10+D11+D12</f>
       </c>
-    </row>
-    <row r="8" spans="6:18" x14ac:dyDescent="0.25">
+      <c r="CX7" s="23" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="8" spans="6:102" x14ac:dyDescent="0.25">
       <c r="F8" s="26" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="L8" s="27">
         <v>1</v>
@@ -3363,13 +3462,16 @@
       <c r="R8" s="27">
         <v>1</v>
       </c>
-    </row>
-    <row r="9" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="CX8" s="26" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="9" spans="1:102" x14ac:dyDescent="0.25">
       <c r="A9" s="26" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="F9" s="26" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="L9" s="28">
         <v>10</v>
@@ -3392,8 +3494,11 @@
       <c r="R9" s="28">
         <v>10</v>
       </c>
-    </row>
-    <row r="10" spans="2:18" x14ac:dyDescent="0.25">
+      <c r="CX9" s="26" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="10" spans="2:102" x14ac:dyDescent="0.25">
       <c r="B10" s="21">
         <f>SUM(L10:R10)</f>
       </c>
@@ -3404,7 +3509,7 @@
         <f>'Rate Tables'!C10</f>
       </c>
       <c r="F10" s="8" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="L10" s="21">
         <f>IF(L$6="","",IF(OR(WEEKDAY(L$6,1)=1,WEEKDAY(L$6,1)=7),0,MIN(8,L9)*L8))</f>
@@ -3427,8 +3532,11 @@
       <c r="R10" s="21">
         <f>IF(R$6="","",IF(OR(WEEKDAY(R$6,1)=1,WEEKDAY(R$6,1)=7),0,MIN(8,R9)*R8))</f>
       </c>
-    </row>
-    <row r="11" spans="2:18" x14ac:dyDescent="0.25">
+      <c r="CX10" s="8" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="11" spans="2:102" x14ac:dyDescent="0.25">
       <c r="B11" s="21">
         <f>SUM(L11:R11)</f>
       </c>
@@ -3439,7 +3547,7 @@
         <f>'Rate Tables'!D10</f>
       </c>
       <c r="F11" s="8" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="L11" s="21">
         <f>IF(L$6="","",IF(WEEKDAY(L$6,1)=1,0,IF(WEEKDAY(L$6,1)=7,L9*L8,MAX(0,L9-8)*L8)))</f>
@@ -3462,8 +3570,11 @@
       <c r="R11" s="21">
         <f>IF(R$6="","",IF(WEEKDAY(R$6,1)=1,0,IF(WEEKDAY(R$6,1)=7,R9*R8,MAX(0,R9-8)*R8)))</f>
       </c>
-    </row>
-    <row r="12" spans="2:18" x14ac:dyDescent="0.25">
+      <c r="CX11" s="8" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="12" spans="2:102" x14ac:dyDescent="0.25">
       <c r="B12" s="21">
         <f>SUM(L12:R12)</f>
       </c>
@@ -3474,7 +3585,7 @@
         <f>'Rate Tables'!E10</f>
       </c>
       <c r="F12" s="8" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="L12" s="21">
         <f>IF(L$6="","",IF(WEEKDAY(L$6,1)=1,L9*L8,0))</f>
@@ -3497,8 +3608,11 @@
       <c r="R12" s="21">
         <f>IF(R$6="","",IF(WEEKDAY(R$6,1)=1,R9*R8,0))</f>
       </c>
-    </row>
-    <row r="13" spans="2:18" x14ac:dyDescent="0.25">
+      <c r="CX12" s="8" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="13" spans="2:102" x14ac:dyDescent="0.25">
       <c r="B13" s="21">
         <f>SUM(L13:R13)</f>
       </c>
@@ -3509,7 +3623,7 @@
         <v>130</v>
       </c>
       <c r="F13" s="8" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="L13" s="19">
         <v>1</v>
@@ -3531,6 +3645,9 @@
       </c>
       <c r="R13" s="19">
         <v>1</v>
+      </c>
+      <c r="CX13" s="8" t="s">
+        <v>64</v>
       </c>
     </row>
     <row r="14" spans="1:11" x14ac:dyDescent="0.25">
@@ -3581,7 +3698,7 @@
   <sheetPr>
     <tabColor rgb="FF1F8A96"/>
   </sheetPr>
-  <dimension ref="A1:R14"/>
+  <dimension ref="A1:CX14"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="28" customWidth="1"/>
@@ -3591,6 +3708,7 @@
     <col min="6" max="10" width="12" customWidth="1"/>
     <col min="11" max="11" width="14" customWidth="1"/>
     <col min="12" max="18" width="7" customWidth="1"/>
+    <col min="102" max="102" width="3" hidden="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="22" customHeight="1" spans="1:18" x14ac:dyDescent="0.25">
@@ -3652,7 +3770,7 @@
         <v>4</v>
       </c>
       <c r="B5" s="6">
-        <v>46269.70988201389</v>
+        <v>46269.71300207176</v>
       </c>
     </row>
     <row r="6" ht="20" customHeight="1" spans="1:18" x14ac:dyDescent="0.25">
@@ -3711,7 +3829,7 @@
         <f>Q6+1</f>
       </c>
     </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:102" x14ac:dyDescent="0.25">
       <c r="A7" s="23" t="s">
         <v>51</v>
       </c>
@@ -3719,11 +3837,14 @@
         <f>G7+H7+I7</f>
       </c>
       <c r="C7" s="23" t="s">
-        <v>60</v>
+        <v>65</v>
       </c>
       <c r="D7" s="25">
         <f>K7</f>
       </c>
+      <c r="F7" s="23" t="s">
+        <v>52</v>
+      </c>
       <c r="G7" s="24">
         <f>B10</f>
       </c>
@@ -3739,10 +3860,13 @@
       <c r="K7" s="25">
         <f>D10+D11+D12</f>
       </c>
-    </row>
-    <row r="8" spans="6:18" x14ac:dyDescent="0.25">
+      <c r="CX7" s="23" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="8" spans="6:102" x14ac:dyDescent="0.25">
       <c r="F8" s="26" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="L8" s="27">
         <v>1</v>
@@ -3765,13 +3889,16 @@
       <c r="R8" s="27">
         <v>1</v>
       </c>
-    </row>
-    <row r="9" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="CX8" s="26" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="9" spans="1:102" x14ac:dyDescent="0.25">
       <c r="A9" s="26" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="F9" s="26" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="L9" s="28">
         <v>10</v>
@@ -3794,8 +3921,11 @@
       <c r="R9" s="28">
         <v>10</v>
       </c>
-    </row>
-    <row r="10" spans="2:18" x14ac:dyDescent="0.25">
+      <c r="CX9" s="26" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="10" spans="2:102" x14ac:dyDescent="0.25">
       <c r="B10" s="21">
         <f>SUM(L10:R10)</f>
       </c>
@@ -3806,7 +3936,7 @@
         <f>'Rate Tables'!C10</f>
       </c>
       <c r="F10" s="8" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="L10" s="21">
         <f>IF(L$6="","",IF(OR(WEEKDAY(L$6,1)=1,WEEKDAY(L$6,1)=7),0,MIN(8,L9)*L8))</f>
@@ -3829,8 +3959,11 @@
       <c r="R10" s="21">
         <f>IF(R$6="","",IF(OR(WEEKDAY(R$6,1)=1,WEEKDAY(R$6,1)=7),0,MIN(8,R9)*R8))</f>
       </c>
-    </row>
-    <row r="11" spans="2:18" x14ac:dyDescent="0.25">
+      <c r="CX10" s="8" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="11" spans="2:102" x14ac:dyDescent="0.25">
       <c r="B11" s="21">
         <f>SUM(L11:R11)</f>
       </c>
@@ -3841,7 +3974,7 @@
         <f>'Rate Tables'!D10</f>
       </c>
       <c r="F11" s="8" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="L11" s="21">
         <f>IF(L$6="","",IF(WEEKDAY(L$6,1)=1,0,IF(WEEKDAY(L$6,1)=7,L9*L8,MAX(0,L9-8)*L8)))</f>
@@ -3864,8 +3997,11 @@
       <c r="R11" s="21">
         <f>IF(R$6="","",IF(WEEKDAY(R$6,1)=1,0,IF(WEEKDAY(R$6,1)=7,R9*R8,MAX(0,R9-8)*R8)))</f>
       </c>
-    </row>
-    <row r="12" spans="2:18" x14ac:dyDescent="0.25">
+      <c r="CX11" s="8" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="12" spans="2:102" x14ac:dyDescent="0.25">
       <c r="B12" s="21">
         <f>SUM(L12:R12)</f>
       </c>
@@ -3876,7 +4012,7 @@
         <f>'Rate Tables'!E10</f>
       </c>
       <c r="F12" s="8" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="L12" s="21">
         <f>IF(L$6="","",IF(WEEKDAY(L$6,1)=1,L9*L8,0))</f>
@@ -3899,8 +4035,11 @@
       <c r="R12" s="21">
         <f>IF(R$6="","",IF(WEEKDAY(R$6,1)=1,R9*R8,0))</f>
       </c>
-    </row>
-    <row r="13" spans="2:18" x14ac:dyDescent="0.25">
+      <c r="CX12" s="8" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="13" spans="2:102" x14ac:dyDescent="0.25">
       <c r="B13" s="21">
         <f>SUM(L13:R13)</f>
       </c>
@@ -3911,7 +4050,7 @@
         <v>130</v>
       </c>
       <c r="F13" s="8" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="L13" s="19">
         <v>1</v>
@@ -3933,6 +4072,9 @@
       </c>
       <c r="R13" s="19">
         <v>1</v>
+      </c>
+      <c r="CX13" s="8" t="s">
+        <v>66</v>
       </c>
     </row>
     <row r="14" spans="1:11" x14ac:dyDescent="0.25">
@@ -4031,41 +4173,41 @@
         <v>4</v>
       </c>
       <c r="B5" s="6">
-        <v>46269.70988201389</v>
+        <v>46269.71300208333</v>
       </c>
     </row>
     <row r="6" ht="20" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A6" s="7" t="s">
-        <v>61</v>
+        <v>67</v>
       </c>
       <c r="B6" s="7" t="s">
-        <v>62</v>
+        <v>68</v>
       </c>
       <c r="C6" s="7" t="s">
-        <v>63</v>
+        <v>69</v>
       </c>
       <c r="D6" s="7" t="s">
-        <v>64</v>
+        <v>70</v>
       </c>
       <c r="E6" s="7" t="s">
-        <v>65</v>
+        <v>71</v>
       </c>
       <c r="F6" s="7" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="G6" s="7" t="s">
-        <v>67</v>
+        <v>73</v>
       </c>
       <c r="H6" s="7" t="s">
-        <v>68</v>
+        <v>74</v>
       </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A7" s="8" t="s">
-        <v>69</v>
+        <v>75</v>
       </c>
       <c r="B7" s="8" t="s">
-        <v>70</v>
+        <v>76</v>
       </c>
       <c r="C7" s="19">
         <v>1</v>
@@ -4167,41 +4309,41 @@
         <v>4</v>
       </c>
       <c r="B5" s="6">
-        <v>46269.70988201389</v>
+        <v>46269.71300208333</v>
       </c>
     </row>
     <row r="6" ht="20" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A6" s="7" t="s">
-        <v>61</v>
+        <v>67</v>
       </c>
       <c r="B6" s="7" t="s">
-        <v>62</v>
+        <v>68</v>
       </c>
       <c r="C6" s="7" t="s">
-        <v>63</v>
+        <v>69</v>
       </c>
       <c r="D6" s="7" t="s">
-        <v>64</v>
+        <v>70</v>
       </c>
       <c r="E6" s="7" t="s">
-        <v>65</v>
+        <v>71</v>
       </c>
       <c r="F6" s="7" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="G6" s="7" t="s">
-        <v>67</v>
+        <v>73</v>
       </c>
       <c r="H6" s="7" t="s">
-        <v>68</v>
+        <v>74</v>
       </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A7" s="8" t="s">
-        <v>71</v>
+        <v>77</v>
       </c>
       <c r="B7" s="8" t="s">
-        <v>70</v>
+        <v>76</v>
       </c>
       <c r="C7" s="19">
         <v>1</v>

</xml_diff>